<commit_message>
Marcar tarea 0.4 como completada (CASF-2016 descomprimido y verificado)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011H6MHrCpLVwMt1Sd8N1Zwv
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="207">
   <si>
     <t xml:space="preserve">CombiLabHUB – Resumen de avance</t>
   </si>
@@ -185,6 +185,9 @@
   </si>
   <si>
     <t xml:space="preserve">Desde PDBbind (requiere registro); dejarlo en SOFTWARE SF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descomprimido en SOFTWARE SF\CASF-2016\CASF-2016 (30.271 archivos verificados contra el .tar.gz; coreset con 285 complejos)</t>
   </si>
   <si>
     <t xml:space="preserve">0.5</t>
@@ -1240,7 +1243,7 @@
       </c>
       <c r="C4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Completada")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"En progreso")</f>
@@ -1248,11 +1251,11 @@
       </c>
       <c r="E4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Pendiente")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">IF(B4=0,0,C4/B4)</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1490,7 +1493,7 @@
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">SUM(C4:C13)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">SUM(D4:D13)</f>
@@ -1498,11 +1501,11 @@
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">SUM(E4:E13)</f>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F14" s="7" t="n">
         <f aca="false">IF(B14=0,0,C14/B14)</f>
-        <v>0.206896551724138</v>
+        <v>0.241379310344828</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1749,25 +1752,31 @@
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="12" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G8" s="12"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="12"/>
+      <c r="H8" s="13" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>46314</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="12" t="s">
@@ -1780,16 +1789,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E10" s="11"/>
       <c r="F10" s="12" t="s">
@@ -1802,19 +1811,19 @@
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>41</v>
@@ -1823,24 +1832,24 @@
       <c r="H11" s="13"/>
       <c r="I11" s="13"/>
       <c r="J11" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>41</v>
@@ -1852,16 +1861,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="12" t="s">
@@ -1874,19 +1883,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F14" s="12" t="s">
         <v>46</v>
@@ -1898,19 +1907,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F15" s="12" t="s">
         <v>46</v>
@@ -1922,19 +1931,19 @@
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F16" s="12" t="s">
         <v>41</v>
@@ -1946,19 +1955,19 @@
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F17" s="12" t="s">
         <v>4</v>
@@ -1967,21 +1976,21 @@
       <c r="H17" s="13"/>
       <c r="I17" s="13"/>
       <c r="J17" s="12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E18" s="11"/>
       <c r="F18" s="12" t="s">
@@ -1991,24 +2000,24 @@
       <c r="H18" s="13"/>
       <c r="I18" s="13"/>
       <c r="J18" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>46</v>
@@ -2020,19 +2029,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F20" s="12" t="s">
         <v>46</v>
@@ -2044,19 +2053,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F21" s="12" t="s">
         <v>46</v>
@@ -2068,19 +2077,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F22" s="12" t="s">
         <v>46</v>
@@ -2092,19 +2101,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F23" s="12" t="s">
         <v>46</v>
@@ -2116,19 +2125,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F24" s="12" t="s">
         <v>46</v>
@@ -2140,19 +2149,19 @@
     </row>
     <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F25" s="12" t="s">
         <v>46</v>
@@ -2161,24 +2170,24 @@
       <c r="H25" s="13"/>
       <c r="I25" s="13"/>
       <c r="J25" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>46</v>
@@ -2190,19 +2199,19 @@
     </row>
     <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F27" s="12" t="s">
         <v>46</v>
@@ -2214,19 +2223,19 @@
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F28" s="12" t="s">
         <v>46</v>
@@ -2238,19 +2247,19 @@
     </row>
     <row r="29" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F29" s="12" t="s">
         <v>46</v>
@@ -2259,24 +2268,24 @@
       <c r="H29" s="13"/>
       <c r="I29" s="13"/>
       <c r="J29" s="12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F30" s="12" t="s">
         <v>46</v>
@@ -2288,16 +2297,16 @@
     </row>
     <row r="31" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E31" s="11"/>
       <c r="F31" s="12" t="s">
@@ -2310,19 +2319,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F32" s="12" t="s">
         <v>46</v>
@@ -2334,19 +2343,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F33" s="12" t="s">
         <v>46</v>
@@ -2411,12 +2420,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2424,34 +2433,34 @@
         <v>19</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2462,13 +2471,13 @@
         <v>1</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
@@ -2488,13 +2497,13 @@
         <v>2</v>
       </c>
       <c r="C6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>151</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>150</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -2514,13 +2523,13 @@
         <v>3</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
@@ -2540,13 +2549,13 @@
         <v>4</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
@@ -2566,13 +2575,13 @@
         <v>5</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
@@ -2592,13 +2601,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
@@ -2618,13 +2627,13 @@
         <v>7</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
@@ -2644,13 +2653,13 @@
         <v>8</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -2670,13 +2679,13 @@
         <v>9</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
@@ -2696,13 +2705,13 @@
         <v>10</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -2722,10 +2731,10 @@
         <v>1</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="12"/>
@@ -2746,10 +2755,10 @@
         <v>2</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="12"/>
@@ -2770,13 +2779,13 @@
         <v>3</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
@@ -2796,13 +2805,13 @@
         <v>4</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
@@ -2822,13 +2831,13 @@
         <v>5</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2848,13 +2857,13 @@
         <v>6</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2874,13 +2883,13 @@
         <v>7</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2900,11 +2909,11 @@
         <v>1</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
@@ -2924,11 +2933,11 @@
         <v>2</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2948,11 +2957,11 @@
         <v>3</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D24" s="11"/>
       <c r="E24" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2972,11 +2981,11 @@
         <v>4</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D25" s="11"/>
       <c r="E25" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
@@ -2996,11 +3005,11 @@
         <v>5</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D26" s="11"/>
       <c r="E26" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
@@ -3020,11 +3029,11 @@
         <v>6</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D27" s="11"/>
       <c r="E27" s="11" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
@@ -3044,11 +3053,11 @@
         <v>7</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D28" s="11"/>
       <c r="E28" s="11" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F28" s="12"/>
       <c r="G28" s="12"/>
@@ -3068,10 +3077,10 @@
         <v>8</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E29" s="11"/>
       <c r="F29" s="12"/>
@@ -3092,11 +3101,11 @@
         <v>9</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D30" s="11"/>
       <c r="E30" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
@@ -3116,11 +3125,11 @@
         <v>10</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D31" s="11"/>
       <c r="E31" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
@@ -3134,7 +3143,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar etapa 0: 0.3 completada, 0.2 en progreso, 0.5 pendiente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011H6MHrCpLVwMt1Sd8N1Zwv
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="210">
   <si>
     <t xml:space="preserve">CombiLabHUB – Resumen de avance</t>
   </si>
@@ -166,37 +166,46 @@
     <t xml:space="preserve">Indicar si hay NVIDIA y modelo (Dynaformer, PIGNet2, HAC-Net la necesitan)</t>
   </si>
   <si>
+    <t xml:space="preserve">Hay GPU NVIDIA con driver de estación de trabajo (RTX/Quadro) 573.44 (soporta CUDA 12.8). Falta confirmar el modelo exacto (Administrador de tareas &gt; Rendimiento &gt; GPU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liberar espacio en disco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~100 GB, o instalar por tandas y borrar entornos probados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">284 GB libres en el disco (más que los ~100 GB necesarios)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descargar CASF-2016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desde PDBbind (requiere registro); dejarlo en SOFTWARE SF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descomprimido en SOFTWARE SF\CASF-2016\CASF-2016 (30.271 archivos verificados contra el .tar.gz; coreset con 285 complejos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habilitar dominios (opcional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conda.anaconda.org, zenodo.org, figshare.com, drive.google.com, onedrive.live.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">0.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liberar espacio en disco</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~100 GB, o instalar por tandas y borrar entornos probados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descargar CASF-2016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desde PDBbind (requiere registro); dejarlo en SOFTWARE SF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descomprimido en SOFTWARE SF\CASF-2016\CASF-2016 (30.271 archivos verificados contra el .tar.gz; coreset con 285 complejos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Habilitar dominios (opcional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">conda.anaconda.org, zenodo.org, figshare.com, drive.google.com, onedrive.live.com</t>
+    <t xml:space="preserve">Probado el 19/10/2026: los 5 dominios están bloqueados. Se habilitan en claude.ai &gt; Settings &gt; Capabilities (lo hace el usuario)</t>
   </si>
   <si>
     <t xml:space="preserve">1.1</t>
@@ -1243,19 +1252,19 @@
       </c>
       <c r="C4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Completada")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"En progreso")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Pendiente")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">IF(B4=0,0,C4/B4)</f>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1493,19 +1502,19 @@
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">SUM(C4:C13)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">SUM(D4:D13)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">SUM(E4:E13)</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F14" s="7" t="n">
         <f aca="false">IF(B14=0,0,C14/B14)</f>
-        <v>0.241379310344828</v>
+        <v>0.275862068965517</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1708,12 +1717,16 @@
       </c>
       <c r="E6" s="11"/>
       <c r="F6" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="12"/>
+      <c r="H6" s="13" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I6" s="13"/>
+      <c r="J6" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
@@ -1730,25 +1743,31 @@
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="12" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G7" s="12"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="12"/>
+      <c r="H7" s="13" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>46314</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="12" t="s">
@@ -1762,43 +1781,45 @@
         <v>46314</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="13"/>
       <c r="I9" s="13"/>
-      <c r="J9" s="12"/>
+      <c r="J9" s="12" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E10" s="11"/>
       <c r="F10" s="12" t="s">
@@ -1811,19 +1832,19 @@
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>41</v>
@@ -1832,24 +1853,24 @@
       <c r="H11" s="13"/>
       <c r="I11" s="13"/>
       <c r="J11" s="12" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>41</v>
@@ -1861,16 +1882,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="12" t="s">
@@ -1883,22 +1904,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G14" s="12"/>
       <c r="H14" s="13"/>
@@ -1907,22 +1928,22 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G15" s="12"/>
       <c r="H15" s="13"/>
@@ -1931,19 +1952,19 @@
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F16" s="12" t="s">
         <v>41</v>
@@ -1955,19 +1976,19 @@
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F17" s="12" t="s">
         <v>4</v>
@@ -1976,21 +1997,21 @@
       <c r="H17" s="13"/>
       <c r="I17" s="13"/>
       <c r="J17" s="12" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E18" s="11"/>
       <c r="F18" s="12" t="s">
@@ -2000,27 +2021,27 @@
       <c r="H18" s="13"/>
       <c r="I18" s="13"/>
       <c r="J18" s="12" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G19" s="12"/>
       <c r="H19" s="13"/>
@@ -2029,22 +2050,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G20" s="12"/>
       <c r="H20" s="13"/>
@@ -2053,22 +2074,22 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G21" s="12"/>
       <c r="H21" s="13"/>
@@ -2077,22 +2098,22 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G22" s="12"/>
       <c r="H22" s="13"/>
@@ -2101,22 +2122,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G23" s="12"/>
       <c r="H23" s="13"/>
@@ -2125,22 +2146,22 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G24" s="12"/>
       <c r="H24" s="13"/>
@@ -2149,48 +2170,48 @@
     </row>
     <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="13"/>
       <c r="I25" s="13"/>
       <c r="J25" s="12" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G26" s="12"/>
       <c r="H26" s="13"/>
@@ -2199,22 +2220,22 @@
     </row>
     <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G27" s="12"/>
       <c r="H27" s="13"/>
@@ -2223,22 +2244,22 @@
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G28" s="12"/>
       <c r="H28" s="13"/>
@@ -2247,48 +2268,48 @@
     </row>
     <row r="29" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G29" s="12"/>
       <c r="H29" s="13"/>
       <c r="I29" s="13"/>
       <c r="J29" s="12" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G30" s="12"/>
       <c r="H30" s="13"/>
@@ -2297,20 +2318,20 @@
     </row>
     <row r="31" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E31" s="11"/>
       <c r="F31" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G31" s="12"/>
       <c r="H31" s="13"/>
@@ -2319,22 +2340,22 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G32" s="12"/>
       <c r="H32" s="13"/>
@@ -2343,22 +2364,22 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G33" s="12"/>
       <c r="H33" s="13"/>
@@ -2420,12 +2441,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2433,34 +2454,34 @@
         <v>19</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2471,13 +2492,13 @@
         <v>1</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
@@ -2497,13 +2518,13 @@
         <v>2</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -2523,13 +2544,13 @@
         <v>3</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
@@ -2549,13 +2570,13 @@
         <v>4</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
@@ -2575,13 +2596,13 @@
         <v>5</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
@@ -2601,13 +2622,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
@@ -2627,13 +2648,13 @@
         <v>7</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
@@ -2653,13 +2674,13 @@
         <v>8</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -2679,13 +2700,13 @@
         <v>9</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
@@ -2705,13 +2726,13 @@
         <v>10</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -2731,10 +2752,10 @@
         <v>1</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="12"/>
@@ -2755,10 +2776,10 @@
         <v>2</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="12"/>
@@ -2779,13 +2800,13 @@
         <v>3</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
@@ -2805,13 +2826,13 @@
         <v>4</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
@@ -2831,13 +2852,13 @@
         <v>5</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2857,13 +2878,13 @@
         <v>6</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2883,13 +2904,13 @@
         <v>7</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2909,11 +2930,11 @@
         <v>1</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="11" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
@@ -2933,11 +2954,11 @@
         <v>2</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="11" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2957,11 +2978,11 @@
         <v>3</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D24" s="11"/>
       <c r="E24" s="11" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2981,11 +3002,11 @@
         <v>4</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D25" s="11"/>
       <c r="E25" s="11" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
@@ -3005,11 +3026,11 @@
         <v>5</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D26" s="11"/>
       <c r="E26" s="11" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
@@ -3029,11 +3050,11 @@
         <v>6</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D27" s="11"/>
       <c r="E27" s="11" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
@@ -3053,11 +3074,11 @@
         <v>7</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D28" s="11"/>
       <c r="E28" s="11" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F28" s="12"/>
       <c r="G28" s="12"/>
@@ -3077,10 +3098,10 @@
         <v>8</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E29" s="11"/>
       <c r="F29" s="12"/>
@@ -3101,11 +3122,11 @@
         <v>9</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D30" s="11"/>
       <c r="E30" s="11" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
@@ -3125,11 +3146,11 @@
         <v>10</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D31" s="11"/>
       <c r="E31" s="11" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
@@ -3143,7 +3164,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Marcar tarea 0.2 como completada (GPU NVIDIA Quadro P620)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011H6MHrCpLVwMt1Sd8N1Zwv
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -166,7 +166,7 @@
     <t xml:space="preserve">Indicar si hay NVIDIA y modelo (Dynaformer, PIGNet2, HAC-Net la necesitan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hay GPU NVIDIA con driver de estación de trabajo (RTX/Quadro) 573.44 (soporta CUDA 12.8). Falta confirmar el modelo exacto (Administrador de tareas &gt; Rendimiento &gt; GPU)</t>
+    <t xml:space="preserve">NVIDIA Quadro P620 (Pascal, 4 GB VRAM, compute 6.1), driver 573.44 + Intel UHD integrada; 31,6 GB RAM. Usar builds de PyTorch cu118/cu126 (las cu128 no soportan Pascal). 4 GB limita a las SF pesadas del Nivel 3</t>
   </si>
   <si>
     <t xml:space="preserve">0.3</t>
@@ -1252,11 +1252,11 @@
       </c>
       <c r="C4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Completada")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"En progreso")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Pendiente")</f>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">IF(B4=0,0,C4/B4)</f>
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1502,11 +1502,11 @@
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">SUM(C4:C13)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">SUM(D4:D13)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">SUM(E4:E13)</f>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="F14" s="7" t="n">
         <f aca="false">IF(B14=0,0,C14/B14)</f>
-        <v>0.275862068965517</v>
+        <v>0.310344827586207</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1717,13 +1717,15 @@
       </c>
       <c r="E6" s="11"/>
       <c r="F6" s="12" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="13" t="n">
         <v>46314</v>
       </c>
-      <c r="I6" s="13"/>
+      <c r="I6" s="13" t="n">
+        <v>46314</v>
+      </c>
       <c r="J6" s="12" t="s">
         <v>46</v>
       </c>

</xml_diff>

<commit_message>
Marcar tarea 0.5 como completada; etapa 0 terminada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011H6MHrCpLVwMt1Sd8N1Zwv
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -202,58 +202,58 @@
     <t xml:space="preserve">conda.anaconda.org, zenodo.org, figshare.com, drive.google.com, onedrive.live.com</t>
   </si>
   <si>
+    <t xml:space="preserve">Verificado 19/10/2026: conda.anaconda.org, zenodo.org, figshare.com, drive.google.com y onedrive.live.com accesibles desde la nube</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extraer tabla de 49 SF del PPTX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scoring_functions_descargadas.xlsx (ES/EN/PT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Investigar 7 columnas extra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dataset, tamaño, tipo, algoritmo, descriptores, feature selection, algoritmo de selección + fuente y confianza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33 Alta, 8 Media, 8 Baja confianza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descargar repos de las 49 SF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funciones_Score_Tabla1/ + INDICE_funciones_score.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descargar SF de Su et al. 2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vina, ΔVinaRF20, vina4dv en Funciones_Score_Su2018/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendientes de descarga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAAP y LigityScore (GitLab); MSSDTA sin código público</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Probado el 19/10/2026: los 5 dominios están bloqueados. Se habilitan en claude.ai &gt; Settings &gt; Capabilities (lo hace el usuario)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extraer tabla de 49 SF del PPTX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scoring_functions_descargadas.xlsx (ES/EN/PT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Investigar 7 columnas extra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset, tamaño, tipo, algoritmo, descriptores, feature selection, algoritmo de selección + fuente y confianza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33 Alta, 8 Media, 8 Baja confianza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descargar repos de las 49 SF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Funciones_Score_Tabla1/ + INDICE_funciones_score.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descargar SF de Su et al. 2019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vina, ΔVinaRF20, vina4dv en Funciones_Score_Su2018/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pendientes de descarga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAAP y LigityScore (GitLab); MSSDTA sin código público</t>
   </si>
   <si>
     <t xml:space="preserve">2.4</t>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Completada")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"En progreso")</f>
@@ -1260,11 +1260,11 @@
       </c>
       <c r="E4" s="4" t="n">
         <f aca="false">COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Pendiente")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">IF(B4=0,0,C4/B4)</f>
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">SUM(C4:C13)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">SUM(D4:D13)</f>
@@ -1510,11 +1510,11 @@
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">SUM(E4:E13)</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F14" s="7" t="n">
         <f aca="false">IF(B14=0,0,C14/B14)</f>
-        <v>0.310344827586207</v>
+        <v>0.344827586206897</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1801,27 +1801,31 @@
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="12"/>
+      <c r="H9" s="13" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>46314</v>
+      </c>
+      <c r="J9" s="12" t="s">
         <v>58</v>
-      </c>
-      <c r="G9" s="12"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="12" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>61</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>62</v>
       </c>
       <c r="E10" s="11"/>
       <c r="F10" s="12" t="s">
@@ -1834,19 +1838,19 @@
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="11" t="s">
-        <v>65</v>
-      </c>
       <c r="E11" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>41</v>
@@ -1855,24 +1859,24 @@
       <c r="H11" s="13"/>
       <c r="I11" s="13"/>
       <c r="J11" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="11" t="s">
-        <v>69</v>
-      </c>
       <c r="E12" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>41</v>
@@ -1884,16 +1888,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>71</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>72</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="12" t="s">
@@ -1906,22 +1910,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="E14" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>75</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>58</v>
       </c>
       <c r="G14" s="12"/>
       <c r="H14" s="13"/>
@@ -1942,10 +1946,10 @@
         <v>78</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G15" s="12"/>
       <c r="H15" s="13"/>
@@ -1966,7 +1970,7 @@
         <v>81</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F16" s="12" t="s">
         <v>41</v>
@@ -2043,7 +2047,7 @@
         <v>93</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G19" s="12"/>
       <c r="H19" s="13"/>
@@ -2067,7 +2071,7 @@
         <v>82</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G20" s="12"/>
       <c r="H20" s="13"/>
@@ -2091,7 +2095,7 @@
         <v>82</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G21" s="12"/>
       <c r="H21" s="13"/>
@@ -2115,7 +2119,7 @@
         <v>97</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G22" s="12"/>
       <c r="H22" s="13"/>
@@ -2139,7 +2143,7 @@
         <v>97</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G23" s="12"/>
       <c r="H23" s="13"/>
@@ -2163,7 +2167,7 @@
         <v>82</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G24" s="12"/>
       <c r="H24" s="13"/>
@@ -2187,7 +2191,7 @@
         <v>112</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="13"/>
@@ -2213,7 +2217,7 @@
         <v>109</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G26" s="12"/>
       <c r="H26" s="13"/>
@@ -2237,7 +2241,7 @@
         <v>114</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G27" s="12"/>
       <c r="H27" s="13"/>
@@ -2261,7 +2265,7 @@
         <v>117</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G28" s="12"/>
       <c r="H28" s="13"/>
@@ -2285,7 +2289,7 @@
         <v>126</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G29" s="12"/>
       <c r="H29" s="13"/>
@@ -2311,7 +2315,7 @@
         <v>109</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G30" s="12"/>
       <c r="H30" s="13"/>
@@ -2333,7 +2337,7 @@
       </c>
       <c r="E31" s="11"/>
       <c r="F31" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G31" s="12"/>
       <c r="H31" s="13"/>
@@ -2357,7 +2361,7 @@
         <v>128</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G32" s="12"/>
       <c r="H32" s="13"/>
@@ -2381,7 +2385,7 @@
         <v>117</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G33" s="12"/>
       <c r="H33" s="13"/>

</xml_diff>

<commit_message>
Add OnionNet-2 plugin: install guide, batch prediction, Dockerfile and 1a30 test
- predict_onionnet2.py: reuses the authors' feature code, converts .mol2/.sdf
  ligands with Open Babel and loads the 885 MB model once
- test_1a30.py: features vs reference, authors' sample 1a30 (5.4568) and
  CASF-2016 1a30 (5.8866); documents the effect of crystallographic waters
- environment.yml: Python 3.8, Open Babel 3.1.1, TensorFlow 2.3.4 CPU,
  scikit-learn 0.22.1 (Windows wheels checked)
- Dockerfile: pinned commit 79e84dd, model from Zenodo with MD5 check
- demo_onionnet2.bat and INSTALL.md
- docs: project sheet updated (OnionNet-2 installed and running)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G3fKs4e1rFzK3T3x5jhdx7
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1756,7 +1756,7 @@
       <c r="I21" s="29" t="n"/>
       <c r="J21" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: hechos ET-Score y GB-Score (environment.yml + Dockerfile con commit y MD5 fijados); faltan 8 del Nivel 1</t>
+          <t>19/10/2026: hechos ET-Score, GB-Score y OnionNet-2 (environment.yml + Dockerfile con commit y MD5 fijados); faltan 7 del Nivel 1</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       <c r="I23" s="29" t="n"/>
       <c r="J23" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score y GB-Score (en inglés)</t>
+          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score, GB-Score y OnionNet-2 (en inglés)</t>
         </is>
       </c>
     </row>
@@ -1944,13 +1944,19 @@
       </c>
       <c r="F26" s="28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="G26" s="28" t="n"/>
-      <c r="H26" s="29" t="n"/>
+      <c r="H26" s="29" t="n">
+        <v>46314</v>
+      </c>
       <c r="I26" s="29" t="n"/>
-      <c r="J26" s="28" t="n"/>
+      <c r="J26" s="28" t="inlineStr">
+        <is>
+          <t>19/10/2026: OnionNet-2 pasa el test con 1a30 (pKd 5.4568 con archivos de los autores, 5.8866 con CASF-2016). Falta SFCNN</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="26.25" customHeight="1" s="17">
       <c r="A27" s="27" t="inlineStr">
@@ -2430,7 +2436,7 @@
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>Modelo en Zenodo</t>
+          <t>62shell_saved-model.h5 (Zenodo 10728089, 885 MB)</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
@@ -2438,15 +2444,29 @@
           <t>TensorFlow CPU</t>
         </is>
       </c>
-      <c r="F7" s="28" t="n"/>
-      <c r="G7" s="28" t="n"/>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H7" s="30" t="n"/>
-      <c r="I7" s="30" t="n"/>
+      <c r="I7" s="30" t="n">
+        <v>0.864</v>
+      </c>
       <c r="J7" s="31">
         <f>IF(AND(ISNUMBER(H7),ISNUMBER(I7)),H7-I7,"")</f>
         <v/>
       </c>
-      <c r="K7" s="28" t="n"/>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>19/10/2026: test 1a30 PASS. TensorFlow 2.3.4 CPU + sklearn 0.22.1 + Open Babel (ligando .mol2 -&gt; .pdb). Las aguas cristalográficas del PDB cambian la predicción (con aguas 5.4568, CASF sin aguas 5.8866): definir qué archivos usar para el PCC. Eaves et al. reproducen PCC 0.851. Plugin: plugins/onionnet2</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="17">
       <c r="A8" s="27" t="n">

</xml_diff>

<commit_message>
Add Sfcnn plugin: install guide, batch prediction, Dockerfile and 1a30 test
- test_1a30.py: 1a30 pKd 5.4721 equals the authors' Sfcnn_2016_test.csv;
  the 74 docking poses match the authors' test/output2 (max diff 0.0007)
- predict_sfcnn.py: batch prediction with the authors' predict.py
  (build_model() loads the weights from the current folder)
- environment.yml: Python 3.8, Open Babel 3.1.1, TensorFlow 2.3.4 CPU
- Dockerfile: pinned commit 30ba8f0, weights MD5 check
- demo_sfcnn.bat and INSTALL.md
- docs: project sheet updated (Sfcnn installed and running, task 5.2 done)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G3fKs4e1rFzK3T3x5jhdx7
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1756,7 +1756,7 @@
       <c r="I21" s="29" t="n"/>
       <c r="J21" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: hechos ET-Score, GB-Score y OnionNet-2 (environment.yml + Dockerfile con commit y MD5 fijados); faltan 7 del Nivel 1</t>
+          <t>19/10/2026: hechos ET-Score, GB-Score, OnionNet-2 y Sfcnn (environment.yml + Dockerfile con commit y MD5 fijados); faltan 6 del Nivel 1</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       <c r="I23" s="29" t="n"/>
       <c r="J23" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score, GB-Score y OnionNet-2 (en inglés)</t>
+          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score, GB-Score, OnionNet-2 y Sfcnn (en inglés)</t>
         </is>
       </c>
     </row>
@@ -1944,17 +1944,19 @@
       </c>
       <c r="F26" s="28" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G26" s="28" t="n"/>
       <c r="H26" s="29" t="n">
         <v>46314</v>
       </c>
-      <c r="I26" s="29" t="n"/>
+      <c r="I26" s="29" t="n">
+        <v>46314</v>
+      </c>
       <c r="J26" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: OnionNet-2 pasa el test con 1a30 (pKd 5.4568 con archivos de los autores, 5.8866 con CASF-2016). Falta SFCNN</t>
+          <t>19/10/2026: OnionNet-2 (pKd 1a30 5.4568 con archivos de los autores / 5.8866 CASF) y Sfcnn (5.4721, igual a los autores; 74 poses de docking iguales) pasan el test con 1a30</t>
         </is>
       </c>
     </row>
@@ -2482,23 +2484,37 @@
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>Pesos en el repo</t>
+          <t>weights_22_112-0.0083.h5 (en el repo, 5.5 MB)</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>TensorFlow + OpenBabel</t>
-        </is>
-      </c>
-      <c r="F8" s="28" t="n"/>
-      <c r="G8" s="28" t="n"/>
+          <t>TensorFlow 2.3 CPU + Open Babel 3.1</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H8" s="30" t="n"/>
-      <c r="I8" s="30" t="n"/>
+      <c r="I8" s="30" t="n">
+        <v>0.793</v>
+      </c>
       <c r="J8" s="31">
         <f>IF(AND(ISNUMBER(H8),ISNUMBER(I8)),H8-I8,"")</f>
         <v/>
       </c>
-      <c r="K8" s="28" t="n"/>
+      <c r="K8" s="28" t="inlineStr">
+        <is>
+          <t>19/10/2026: test 1a30 PASS: pKd 5.4721 idéntico a Sfcnn_2016_test.csv de los autores y 74 poses de docking iguales a test/output2 (dif. máx 0.0007). build_model() carga los pesos desde la carpeta actual. Eaves et al. reproducen PCC 0.789. Plugin: plugins/sfcnn</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="17">
       <c r="A9" s="27" t="n">

</xml_diff>

<commit_message>
Add PLANET plugin: install guide, batch prediction, Dockerfile and 1a30 test
- predict_planet.py: scores a folder of complexes with the authors'
  PlanetEstimator; falls back to .mol2 when RDKit cannot sanitize the .sdf
- test_1a30.py: authors' prepared 1a30 (core.tar.bz2) 5.8930 and CASF-2016
  files 5.6216; documents the input-format sensitivity
- environment.yml: Python 3.11, PyTorch 2.2.2, RDKit 2023.9.5 (Windows
  wheels checked); Dockerfile with CPU-only PyTorch and MD5 checks
- demo_planet.bat and INSTALL.md (demo/result.csv is from the 2022 model)
- docs: project sheet updated (PLANET installed and running)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G3fKs4e1rFzK3T3x5jhdx7
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1756,7 +1756,7 @@
       <c r="I21" s="29" t="n"/>
       <c r="J21" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: hechos ET-Score, GB-Score, OnionNet-2 y Sfcnn (environment.yml + Dockerfile con commit y MD5 fijados); faltan 6 del Nivel 1</t>
+          <t>19/10/2026: hechos ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET (environment.yml + Dockerfile con commit y MD5 fijados); faltan 5 del Nivel 1</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       <c r="I23" s="29" t="n"/>
       <c r="J23" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score, GB-Score, OnionNet-2 y Sfcnn (en inglés)</t>
+          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET (en inglés)</t>
         </is>
       </c>
     </row>
@@ -1988,13 +1988,19 @@
       </c>
       <c r="F27" s="28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="G27" s="28" t="n"/>
-      <c r="H27" s="29" t="n"/>
+      <c r="H27" s="29" t="n">
+        <v>46314</v>
+      </c>
       <c r="I27" s="29" t="n"/>
-      <c r="J27" s="28" t="n"/>
+      <c r="J27" s="28" t="inlineStr">
+        <is>
+          <t>19/10/2026: PLANET pasa el test con 1a30 (5.8930 con archivos de los autores, 5.6216 con CASF). Faltan egGNN, GIGN, EHIGN-PLA, saCNN, DEAttentionDTA</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="26.25" customHeight="1" s="17">
       <c r="A28" s="27" t="inlineStr">
@@ -2530,23 +2536,37 @@
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>PLANET.param en el repo</t>
+          <t>PLANET.param (en el repo, 18.5 MB) + core.tar.bz2 (core set preparado por los autores)</t>
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr">
         <is>
-          <t>PyTorch + RDKit</t>
-        </is>
-      </c>
-      <c r="F9" s="28" t="n"/>
-      <c r="G9" s="28" t="n"/>
+          <t>PyTorch 2.2 + RDKit 2023.9 (Python 3.11)</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H9" s="30" t="n"/>
-      <c r="I9" s="30" t="n"/>
+      <c r="I9" s="30" t="n">
+        <v>0.824</v>
+      </c>
       <c r="J9" s="31">
         <f>IF(AND(ISNUMBER(H9),ISNUMBER(I9)),H9-I9,"")</f>
         <v/>
       </c>
-      <c r="K9" s="28" t="n"/>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>19/10/2026: test 1a30 PASS (5.8930 con core.tar.bz2 de los autores; 5.6216 con CASF .mol2). El .sdf de CASF de 1a30 no lo lee RDKit: usar core.tar.bz2 de los autores. demo/result.csv es de 2022 (modelo viejo), no sirve de referencia. Plugin: plugins/planet</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="17">
       <c r="A10" s="27" t="n">

</xml_diff>

<commit_message>
Add egGNN plugin: install guide, batch prediction, Dockerfile and 1a30 test
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XW5brJzmAKak8eH6gtoyTm
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etapas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estado SF" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Etapas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Estado SF" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Etapas'!$A$4:$J$33</definedName>
@@ -1756,7 +1756,7 @@
       <c r="I21" s="29" t="n"/>
       <c r="J21" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: hechos ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET (environment.yml + Dockerfile con commit y MD5 fijados); faltan 5 del Nivel 1</t>
+          <t>19/10/2026: hechos ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET (environment.yml + Dockerfile con commit y MD5 fijados) | 20/10/2026: egGNN hecho; faltan 4 del Nivel 1</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       <c r="I23" s="29" t="n"/>
       <c r="J23" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET (en inglés)</t>
+          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET (en inglés) | 20/10/2026: egGNN</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       <c r="I27" s="29" t="n"/>
       <c r="J27" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: PLANET pasa el test con 1a30 (5.8930 con archivos de los autores, 5.6216 con CASF). Faltan egGNN, GIGN, EHIGN-PLA, saCNN, DEAttentionDTA</t>
+          <t>19/10/2026: PLANET pasa el test con 1a30 (5.8930 con archivos de los autores, 5.6216 con CASF) | 20/10/2026: egGNN pasa el test con 1a30 (5.1040 con pocket, igual a Eaves et al.). Faltan GIGN, EHIGN-PLA, saCNN, DEAttentionDTA</t>
         </is>
       </c>
     </row>
@@ -2582,23 +2582,35 @@
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>Checkpoint en el repo</t>
+          <t>16-8596.sav (en el repo, 11.7 MB; usado por el pipeline de los autores)</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr">
         <is>
-          <t>SMILES + PDB</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="n"/>
-      <c r="G10" s="28" t="n"/>
+          <t>PyTorch 2.2 + DGL 2.2.1 + dgllife 0.3.2 + RDKit (Python 3.10)</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H10" s="30" t="n"/>
       <c r="I10" s="30" t="n"/>
       <c r="J10" s="31">
         <f>IF(AND(ISNUMBER(H10),ISNUMBER(I10)),H10-I10,"")</f>
         <v/>
       </c>
-      <c r="K10" s="28" t="n"/>
+      <c r="K10" s="28" t="inlineStr">
+        <is>
+          <t>20/10/2026: test 1a30 PASS (pKd 5.1040 con pocket, idéntico a Eaves et al.; 6.5326 con proteína completa). Usar _pocket.pdb: con la proteína completa Eaves obtiene PCC 0.071, con el pocket 0.669 (no reproduce el 0.86 del artículo). Ligando como SMILES desde el .mol2. El checkpoint es un modelo pickleado con clases __main__.*: el wrapper las redirige. Plugin: plugins/eggnn</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="17">
       <c r="A11" s="27" t="n">
@@ -3224,6 +3236,7 @@
       </c>
       <c r="K31" s="28" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="17">
       <c r="A33" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update project sheet: Level 1 complete (10/10 scoring functions pass the 1a30 test)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XW5brJzmAKak8eH6gtoyTm
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1746,17 +1746,19 @@
       </c>
       <c r="F21" s="28" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G21" s="28" t="n"/>
       <c r="H21" s="29" t="n">
         <v>46314</v>
       </c>
-      <c r="I21" s="29" t="n"/>
+      <c r="I21" s="29" t="n">
+        <v>46315</v>
+      </c>
       <c r="J21" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: hechos ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET (environment.yml + Dockerfile con commit y MD5 fijados) | 20/10/2026: egGNN hecho; faltan 4 del Nivel 1</t>
+          <t>19/10/2026: hechos ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET | 20/10/2026: egGNN, GIGN, EHIGN-PLA, saCNN y DEAttentionDTA. Nivel 1 completo (10/10), environment.yml + Dockerfile con commit y MD5 fijados</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1836,7 @@
       <c r="I23" s="29" t="n"/>
       <c r="J23" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: INSTALL.md + test_1a30.py + demo .bat hechos para ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET (en inglés) | 20/10/2026: egGNN</t>
+          <t>19/10/2026: ET-Score, GB-Score, OnionNet-2, Sfcnn y PLANET | 20/10/2026: egGNN, GIGN, EHIGN-PLA, saCNN y DEAttentionDTA. INSTALL.md + test_1a30.py + demo .bat para las 10 SF del Nivel 1 (en inglés)</t>
         </is>
       </c>
     </row>
@@ -1988,17 +1990,19 @@
       </c>
       <c r="F27" s="28" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G27" s="28" t="n"/>
       <c r="H27" s="29" t="n">
         <v>46314</v>
       </c>
-      <c r="I27" s="29" t="n"/>
+      <c r="I27" s="29" t="n">
+        <v>46315</v>
+      </c>
       <c r="J27" s="28" t="inlineStr">
         <is>
-          <t>19/10/2026: PLANET pasa el test con 1a30 (5.8930 con archivos de los autores, 5.6216 con CASF) | 20/10/2026: egGNN pasa el test con 1a30 (5.1040 con pocket, igual a Eaves et al.). Faltan GIGN, EHIGN-PLA, saCNN, DEAttentionDTA</t>
+          <t>19/10/2026: PLANET pasa el test con 1a30 | 20/10/2026: egGNN (5.1040), GIGN (media 5.7230), EHIGN-PLA (media 5.4670), saCNN (5.0950) y DEAttentionDTA (6.2026 CASF / 6.3185 autores) pasan el test con 1a30 en Linux. Falta confirmar en Windows</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2605,9 @@
         </is>
       </c>
       <c r="H10" s="30" t="n"/>
-      <c r="I10" s="30" t="n"/>
+      <c r="I10" s="30" t="n">
+        <v>0.86</v>
+      </c>
       <c r="J10" s="31">
         <f>IF(AND(ISNUMBER(H10),ISNUMBER(I10)),H10-I10,"")</f>
         <v/>
@@ -2626,23 +2632,37 @@
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
-          <t>Pesos en el repo</t>
+          <t>3 modelos en el repo (repeat0-2, .pt)</t>
         </is>
       </c>
       <c r="E11" s="27" t="inlineStr">
         <is>
-          <t>PyTorch</t>
-        </is>
-      </c>
-      <c r="F11" s="28" t="n"/>
-      <c r="G11" s="28" t="n"/>
+          <t>PyTorch 2.2 + PyG 2.5.3 + RDKit + PyMOL + Open Babel (entorno gign, Python 3.10)</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H11" s="30" t="n"/>
-      <c r="I11" s="30" t="n"/>
+      <c r="I11" s="30" t="n">
+        <v>0.84</v>
+      </c>
       <c r="J11" s="31">
         <f>IF(AND(ISNUMBER(H11),ISNUMBER(I11)),H11-I11,"")</f>
         <v/>
       </c>
-      <c r="K11" s="28" t="n"/>
+      <c r="K11" s="28" t="inlineStr">
+        <is>
+          <t>20/10/2026: test 1a30 PASS (modelos 4.3883 / 6.3427 / 6.4380, media 5.7230, igual a los scripts de los autores). Nuestro grafo de 1a30 es idéntico al preparado por los autores (Zenodo 7490623); con sus 285 grafos del core set: PCC 0.844 / 0.843 / 0.832, 0.855 con la media. Pocket con PyMOL a 5 Å + obabel -d. Eaves et al. reproducen PCC 0.85. Plugin: plugins/gign</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="17">
       <c r="A12" s="27" t="n">
@@ -2658,23 +2678,37 @@
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>Pesos en el repo</t>
+          <t>3 modelos en el repo (repeat0-2, .pt)</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr">
         <is>
-          <t>Mismo entorno que GIGN</t>
-        </is>
-      </c>
-      <c r="F12" s="28" t="n"/>
-      <c r="G12" s="28" t="n"/>
+          <t>PyTorch 2.2 + DGL 2.2.1 + RDKit + PyMOL + Open Babel (mismo entorno gign que GIGN)</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H12" s="30" t="n"/>
-      <c r="I12" s="30" t="n"/>
+      <c r="I12" s="30" t="n">
+        <v>0.854</v>
+      </c>
       <c r="J12" s="31">
         <f>IF(AND(ISNUMBER(H12),ISNUMBER(I12)),H12-I12,"")</f>
         <v/>
       </c>
-      <c r="K12" s="28" t="n"/>
+      <c r="K12" s="28" t="inlineStr">
+        <is>
+          <t>20/10/2026: test 1a30 PASS (5.5024 / 5.8087 / 5.0898, media 5.4670, igual a los scripts de los autores). Código para DGL 0.9: copy_src mapeado a copy_u; el modelo modifica el grafo, se recarga por modelo. Falta calcular el PCC del core set. Eaves et al. reproducen PCC 0.851. Plugin: plugins/ehign_pla</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="17">
       <c r="A13" s="27" t="n">
@@ -2690,23 +2724,37 @@
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>Pesos en el repo</t>
+          <t>model.pkl (en el repo, 18.2 MB)</t>
         </is>
       </c>
       <c r="E13" s="27" t="inlineStr">
         <is>
-          <t>moleculekit</t>
-        </is>
-      </c>
-      <c r="F13" s="28" t="n"/>
-      <c r="G13" s="28" t="n"/>
+          <t>PyTorch 2.5 CPU + moleculekit 1.11.5 + pdb2pqr/propka (Python 3.10); sin HTMD</t>
+        </is>
+      </c>
+      <c r="F13" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H13" s="30" t="n"/>
-      <c r="I13" s="30" t="n"/>
+      <c r="I13" s="30" t="n">
+        <v>0.865</v>
+      </c>
       <c r="J13" s="31">
         <f>IF(AND(ISNUMBER(H13),ISNUMBER(I13)),H13-I13,"")</f>
         <v/>
       </c>
-      <c r="K13" s="28" t="n"/>
+      <c r="K13" s="28" t="inlineStr">
+        <is>
+          <t>20/10/2026: test 1a30 PASS (pKd 5.0950, idéntico a Eaves et al.; 3jvr 4.7484 y features iguales a los de los autores). No requiere HTMD (htmd 2.0.6 pide acemd3 no público): se usa moleculekit 1.11.5 con la preparación corregida de Eaves, sin el fallback HTMD/CHARMM. Checkpoint guardado en GPU, se carga en CPU. Eaves et al. reproducen PCC 0.862. Plugin: plugins/sacnn</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="17">
       <c r="A14" s="27" t="n">
@@ -2722,23 +2770,37 @@
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>Pesos en el repo</t>
+          <t>10 modelos Fold 1–10 (en el repo, 89 MB; se promedian)</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr">
         <is>
-          <t>Solo secuencias</t>
-        </is>
-      </c>
-      <c r="F14" s="28" t="n"/>
-      <c r="G14" s="28" t="n"/>
+          <t>PyTorch 2.2 + Open Babel 3.1.1 (Python 3.10)</t>
+        </is>
+      </c>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H14" s="30" t="n"/>
-      <c r="I14" s="30" t="n"/>
+      <c r="I14" s="30" t="n">
+        <v>0.845</v>
+      </c>
       <c r="J14" s="31">
         <f>IF(AND(ISNUMBER(H14),ISNUMBER(I14)),H14-I14,"")</f>
         <v/>
       </c>
-      <c r="K14" s="28" t="n"/>
+      <c r="K14" s="28" t="inlineStr">
+        <is>
+          <t>20/10/2026: test 1a30 PASS (6.3185 con los datos preprocesados de los autores, igual a su kfold_result.csv; 6.2026 con archivos CASF: mismo SMILES y secuencia, pocket CASF 51 vs 56 residuos). Con los datos de los autores reproduce su kfold_result.csv en 278 complejos (PCC 0.853). Los pocket de CASF no tienen cadena: el wrapper asigna cada residuo por número y nombre en orden (A y luego B). Eaves et al. reproducen PCC 0.819. Plugin: plugins/deattentiondta</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="17">
       <c r="A15" s="27" t="n">

</xml_diff>

<commit_message>
Update project sheet: README done, core set runner ready (8.1 in progress)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Etapas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Estado SF" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etapas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estado SF" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Etapas'!$A$4:$J$33</definedName>
@@ -1674,13 +1674,17 @@
       </c>
       <c r="F19" s="28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G19" s="28" t="n"/>
       <c r="H19" s="29" t="n"/>
       <c r="I19" s="29" t="n"/>
-      <c r="J19" s="28" t="n"/>
+      <c r="J19" s="28" t="inlineStr">
+        <is>
+          <t>Superada: el código se subió plugin por plugin al repo temporal (commits del 19 y 20/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="17">
       <c r="A20" s="27" t="inlineStr">
@@ -1868,13 +1872,21 @@
       </c>
       <c r="F24" s="28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G24" s="28" t="n"/>
-      <c r="H24" s="29" t="n"/>
-      <c r="I24" s="29" t="n"/>
-      <c r="J24" s="28" t="n"/>
+      <c r="H24" s="29" t="n">
+        <v>46316</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>46316</v>
+      </c>
+      <c r="J24" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: README.md con estructura, carpetas, uso rápido y cómo agregar una SF</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="26.25" customHeight="1" s="17">
       <c r="A25" s="27" t="inlineStr">
@@ -2110,13 +2122,19 @@
       </c>
       <c r="F30" s="28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="G30" s="28" t="n"/>
-      <c r="H30" s="29" t="n"/>
+      <c r="H30" s="29" t="n">
+        <v>46316</v>
+      </c>
       <c r="I30" s="29" t="n"/>
-      <c r="J30" s="28" t="n"/>
+      <c r="J30" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: tools/run_coreset_level1.bat corre las 10 SF del Nivel 1 sobre el core set y tools/evaluate_casf.py calcula PCC (IC 90% bootstrap), SD, Spearman y RMSE contra CoreSet.dat. Falta ejecutarlo en la PC del laboratorio</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="26.25" customHeight="1" s="17">
       <c r="A31" s="27" t="inlineStr">
@@ -3298,7 +3316,6 @@
       </c>
       <c r="K31" s="28" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="17">
       <c r="A33" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Project sheet: Level 1 core set test reserved for a video recording
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1926,7 +1926,7 @@
       <c r="I25" s="29" t="n"/>
       <c r="J25" s="28" t="inlineStr">
         <is>
-          <t>Primeras a probar | 19/10/2026: ET-Score y GB-Score pasan el test con 1a30 (pKd 5.6837 y 5.6171). Falta correr el core set completo y calcular PCC</t>
+          <t>Primeras a probar | 19/10/2026: ET-Score y GB-Score pasan el test con 1a30 (pKd 5.6837 y 5.6171). Falta correr el core set completo y calcular PCC | 21/10/2026: la corrida del core set completo queda reservada para el video (ver 8.1)</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,11 @@
       <c r="G28" s="28" t="n"/>
       <c r="H28" s="29" t="n"/>
       <c r="I28" s="29" t="n"/>
-      <c r="J28" s="28" t="n"/>
+      <c r="J28" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: se avanza con el Nivel 2 preparando cada SF solo hasta el test con 1a30</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="26.25" customHeight="1" s="17">
       <c r="A29" s="27" t="inlineStr">
@@ -2122,17 +2126,15 @@
       </c>
       <c r="F30" s="28" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G30" s="28" t="n"/>
-      <c r="H30" s="29" t="n">
-        <v>46316</v>
-      </c>
+      <c r="H30" s="29" t="n"/>
       <c r="I30" s="29" t="n"/>
       <c r="J30" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: tools/run_coreset_level1.bat corre las 10 SF del Nivel 1 sobre el core set y tools/evaluate_casf.py calcula PCC (IC 90% bootstrap), SD, Spearman y RMSE contra CoreSet.dat. Falta ejecutarlo en la PC del laboratorio</t>
+          <t>21/10/2026: tools/run_coreset_level1.bat y tools/evaluate_casf.py listos (PCC, IC 90%, SD, Spearman, RMSE vs CoreSet.dat). El test de los 285 complejos del Nivel 1 se va a ejecutar y grabar en un VIDEO; no correrlo antes. El usuario lo quiere hacer de otra manera</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Project sheet: add task 6.2, find out how GraphscoreDTA builds its test complexes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -589,6 +589,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="26.25" customHeight="1" s="17">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -628,19 +629,19 @@
         </is>
       </c>
       <c r="B4" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A4)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A4)</f>
         <v/>
       </c>
       <c r="C4" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A4,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D4" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A4,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E4" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A4,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A4,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F4" s="21">
@@ -655,19 +656,19 @@
         </is>
       </c>
       <c r="B5" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A5)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A5)</f>
         <v/>
       </c>
       <c r="C5" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A5,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A5,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D5" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A5,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A5,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E5" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A5,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A5,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F5" s="21">
@@ -682,19 +683,19 @@
         </is>
       </c>
       <c r="B6" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A6)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A6)</f>
         <v/>
       </c>
       <c r="C6" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A6,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A6,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D6" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A6,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A6,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E6" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A6,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A6,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F6" s="21">
@@ -709,19 +710,19 @@
         </is>
       </c>
       <c r="B7" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A7)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A7)</f>
         <v/>
       </c>
       <c r="C7" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A7,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A7,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D7" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A7,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A7,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E7" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A7,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A7,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F7" s="21">
@@ -736,19 +737,19 @@
         </is>
       </c>
       <c r="B8" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A8)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A8)</f>
         <v/>
       </c>
       <c r="C8" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A8,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A8,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D8" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A8,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A8,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E8" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A8,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A8,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F8" s="21">
@@ -763,19 +764,19 @@
         </is>
       </c>
       <c r="B9" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A9)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A9)</f>
         <v/>
       </c>
       <c r="C9" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A9,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A9,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D9" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A9,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A9,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E9" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A9,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A9,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F9" s="21">
@@ -790,19 +791,19 @@
         </is>
       </c>
       <c r="B10" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A10)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A10)</f>
         <v/>
       </c>
       <c r="C10" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A10,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A10,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D10" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A10,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A10,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E10" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A10,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A10,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F10" s="21">
@@ -817,19 +818,19 @@
         </is>
       </c>
       <c r="B11" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A11)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A11)</f>
         <v/>
       </c>
       <c r="C11" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A11,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A11,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D11" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A11,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A11,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E11" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A11,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A11,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F11" s="21">
@@ -844,19 +845,19 @@
         </is>
       </c>
       <c r="B12" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A12)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A12)</f>
         <v/>
       </c>
       <c r="C12" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A12,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A12,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D12" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A12,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A12,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E12" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A12,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A12,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F12" s="21">
@@ -871,19 +872,19 @@
         </is>
       </c>
       <c r="B13" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$33,A13)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$34,A13)</f>
         <v/>
       </c>
       <c r="C13" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A13,Etapas!$F$5:$F$33,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A13,Etapas!$F$5:$F$34,"Completada")</f>
         <v/>
       </c>
       <c r="D13" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A13,Etapas!$F$5:$F$33,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A13,Etapas!$F$5:$F$34,"En progreso")</f>
         <v/>
       </c>
       <c r="E13" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$33,A13,Etapas!$F$5:$F$33,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$34,A13,Etapas!$F$5:$F$34,"Pendiente")</f>
         <v/>
       </c>
       <c r="F13" s="21">
@@ -918,6 +919,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="17">
       <c r="A16" s="24" t="inlineStr">
         <is>
@@ -1035,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="16" min="1" max="1"/>
@@ -1062,6 +1064,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="17">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -2061,27 +2064,27 @@
     <row r="29" ht="26.25" customHeight="1" s="17">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>7. Pruebas Nivel 3 (pesadas/complicadas)</t>
+          <t>6. Pruebas Nivel 2 (pasos extra)</t>
         </is>
       </c>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>SF del Nivel 3</t>
+          <t>Investigar cómo GraphscoreDTA prepara sus complejos de test</t>
         </is>
       </c>
       <c r="D29" s="27" t="inlineStr">
         <is>
-          <t>PointNet, PIGNet2, Dynaformer, TopoFormer, BAPA, CGraphDTA, EGNA, HydraScreen, RFL-Score, P3-Score</t>
+          <t>Los autores publicaron solo los grafos ya armados de 279 complejos de CASF-2016 (all_in_one_graph_test2016.bin + Vina_terms2016.pkl), no el código que los genera. Averiguar cómo construyen el grafo (átomos del ligando, residuos del pocket, interacciones) y los 6 términos de Vina, para poder preparar 1a30 y complejos nuevos</t>
         </is>
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>6.1, 0.2</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="F29" s="28" t="inlineStr">
@@ -2090,38 +2093,40 @@
         </is>
       </c>
       <c r="G29" s="28" t="n"/>
-      <c r="H29" s="29" t="n"/>
+      <c r="H29" s="29" t="n">
+        <v>46316</v>
+      </c>
       <c r="I29" s="29" t="n"/>
       <c r="J29" s="28" t="inlineStr">
         <is>
-          <t>GPU, licencias (X-Score) o API (HydraScreen)</t>
+          <t>21/10/2026: 1a30, 2zcr, 2zy1, 3ag9, 3bv9 y 3uri no están en el set de los autores. Pistas: artículo (Bioinformatics 2023, btad340) y su material suplementario, repo espejo KailiWang1/GraphscoreDTA, preguntar a los autores (kailiwang@dhu.edu.cn)</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="17">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>8. Evaluación en CASF-2016</t>
+          <t>7. Pruebas Nivel 3 (pesadas/complicadas)</t>
         </is>
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>Calcular PCC por SF</t>
+          <t>SF del Nivel 3</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>Comparar PCC obtenido vs. reportado (hoja Estado SF)</t>
+          <t>PointNet, PIGNet2, Dynaformer, TopoFormer, BAPA, CGraphDTA, EGNA, HydraScreen, RFL-Score, P3-Score</t>
         </is>
       </c>
       <c r="E30" s="27" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.1, 0.2</t>
         </is>
       </c>
       <c r="F30" s="28" t="inlineStr">
@@ -2134,14 +2139,14 @@
       <c r="I30" s="29" t="n"/>
       <c r="J30" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: tools/run_coreset_level1.bat y tools/evaluate_casf.py listos (PCC, IC 90%, SD, Spearman, RMSE vs CoreSet.dat). El test de los 285 complejos del Nivel 1 se va a ejecutar y grabar en un VIDEO; no correrlo antes. El usuario lo quiere hacer de otra manera</t>
+          <t>GPU, licencias (X-Score) o API (HydraScreen)</t>
         </is>
       </c>
     </row>
     <row r="31" ht="26.25" customHeight="1" s="17">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B31" s="27" t="inlineStr">
@@ -2151,15 +2156,19 @@
       </c>
       <c r="C31" s="27" t="inlineStr">
         <is>
-          <t>Usar versiones corregidas de Eaves et al.</t>
+          <t>Calcular PCC por SF</t>
         </is>
       </c>
       <c r="D31" s="27" t="inlineStr">
         <is>
-          <t>17 modelos en github.com/jeavesj</t>
-        </is>
-      </c>
-      <c r="E31" s="27" t="n"/>
+          <t>Comparar PCC obtenido vs. reportado (hoja Estado SF)</t>
+        </is>
+      </c>
+      <c r="E31" s="27" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
       <c r="F31" s="28" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -2168,12 +2177,16 @@
       <c r="G31" s="28" t="n"/>
       <c r="H31" s="29" t="n"/>
       <c r="I31" s="29" t="n"/>
-      <c r="J31" s="28" t="n"/>
+      <c r="J31" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: tools/run_coreset_level1.bat y tools/evaluate_casf.py listos (PCC, IC 90%, SD, Spearman, RMSE vs CoreSet.dat). El test de los 285 complejos del Nivel 1 se va a ejecutar y grabar en un VIDEO; no correrlo antes. El usuario lo quiere hacer de otra manera</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="17">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B32" s="27" t="inlineStr">
@@ -2183,19 +2196,15 @@
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>Informe comparativo</t>
+          <t>Usar versiones corregidas de Eaves et al.</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>Tabla/gráficos de resultados para el laboratorio</t>
-        </is>
-      </c>
-      <c r="E32" s="27" t="inlineStr">
-        <is>
-          <t>8.1</t>
-        </is>
-      </c>
+          <t>17 modelos en github.com/jeavesj</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="n"/>
       <c r="F32" s="28" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -2209,27 +2218,27 @@
     <row r="33" ht="15" customHeight="1" s="17">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B33" s="27" t="inlineStr">
         <is>
-          <t>9. Interfaz</t>
+          <t>8. Evaluación en CASF-2016</t>
         </is>
       </c>
       <c r="C33" s="27" t="inlineStr">
         <is>
-          <t>Interfaz para ejecutar cada SF</t>
+          <t>Informe comparativo</t>
         </is>
       </c>
       <c r="D33" s="27" t="inlineStr">
         <is>
-          <t>UI sobre el CLI de CombiLabHUB</t>
+          <t>Tabla/gráficos de resultados para el laboratorio</t>
         </is>
       </c>
       <c r="E33" s="27" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="F33" s="28" t="inlineStr">
@@ -2241,6 +2250,42 @@
       <c r="H33" s="29" t="n"/>
       <c r="I33" s="29" t="n"/>
       <c r="J33" s="28" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>9. Interfaz</t>
+        </is>
+      </c>
+      <c r="C34" s="27" t="inlineStr">
+        <is>
+          <t>Interfaz para ejecutar cada SF</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>UI sobre el CLI de CombiLabHUB</t>
+        </is>
+      </c>
+      <c r="E34" s="27" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F34" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n"/>
+      <c r="H34" s="29" t="n"/>
+      <c r="I34" s="29" t="n"/>
+      <c r="J34" s="28" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:J33"/>
@@ -2305,6 +2350,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="39" customHeight="1" s="17">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -3318,6 +3364,7 @@
       </c>
       <c r="K31" s="28" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="17">
       <c r="A33" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Level 2 done up to the 1a30 test; CPIScore discarded (incomplete model); update project sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -589,7 +589,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="26.25" customHeight="1" s="17">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -919,7 +918,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="17">
       <c r="A16" s="24" t="inlineStr">
         <is>
@@ -1064,7 +1062,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="17">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -2049,15 +2046,19 @@
       </c>
       <c r="F28" s="28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G28" s="28" t="n"/>
-      <c r="H28" s="29" t="n"/>
-      <c r="I28" s="29" t="n"/>
+      <c r="H28" s="29" t="n">
+        <v>46316</v>
+      </c>
+      <c r="I28" s="29" t="n">
+        <v>46316</v>
+      </c>
       <c r="J28" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: se avanza con el Nivel 2 preparando cada SF solo hasta el test con 1a30</t>
+          <t>21/10/2026: Nivel 2 hasta el test con 1a30: IGModel, ConBAP, HAC-Net, delta_LinF9_XGB y DeepBindGCN PASS; GraphscoreDTA instalada pero sin 1a30 (sin featurizador público, ver 6.2); CPIScore descartada (modelo incompleto). Probado en Linux; falta confirmar los demos en Windows (delta_LinF9_XGB solo por Docker/WSL; HAC-Net necesita internet para ACC2)</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2351,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="39" customHeight="1" s="17">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -2882,19 +2882,37 @@
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>Release de GitHub</t>
-        </is>
-      </c>
-      <c r="E15" s="27" t="n"/>
-      <c r="F15" s="28" t="n"/>
-      <c r="G15" s="28" t="n"/>
+          <t>GitHub release v1.0.0: full_model_out2000_RG.model (MD5 aaa69454…)</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>PyTorch 2.2 + PyG 2.5.3 + RDKit (Python 3.10)</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H15" s="30" t="n"/>
-      <c r="I15" s="30" t="n"/>
+      <c r="I15" s="30" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J15" s="31">
         <f>IF(AND(ISNUMBER(H15),ISNUMBER(I15)),H15-I15,"")</f>
         <v/>
       </c>
-      <c r="K15" s="28" t="n"/>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: test 1a30 PASS (pKd 4.4640, valor propio). El modelo es una red PyG 1.4 pickleada: su GCNConv normaliza por el grado del nodo origen (PyG actual: destino) y el grafo del pocket es dirigido; con la capa actual 1a30 da 6.4782. Se usa una copia exacta de la capa vieja. Plugin: plugins/deepbindgcn</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="17">
       <c r="A16" s="27" t="n">
@@ -2910,19 +2928,37 @@
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>pip HACNet</t>
-        </is>
-      </c>
-      <c r="E16" s="27" t="n"/>
-      <c r="F16" s="28" t="n"/>
-      <c r="G16" s="28" t="n"/>
+          <t>HACNet/parameter_files en el repo (4 .pt) + paquete PyPI HACNet 1.4.3</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>PyTorch 2.2 + PyG 2.5.3 + Open Babel + PyMOL; cargas EqEq: servicio web ACC2 o ChargeFW2 local (Docker)</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H16" s="30" t="n"/>
-      <c r="I16" s="30" t="n"/>
+      <c r="I16" s="30" t="n">
+        <v>0.846</v>
+      </c>
       <c r="J16" s="31">
         <f>IF(AND(ISNUMBER(H16),ISNUMBER(I16)),H16-I16,"")</f>
         <v/>
       </c>
-      <c r="K16" s="28" t="n"/>
+      <c r="K16" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: test 1a30 PASS con ChargeFW2 3.0.0 (pKd 4.9114, valor propio). El servidor de cargas original ya no existe: se usa ACC2 (internet) o ChargeFW2 compilado en Docker. Hallazgo: el notebook/fork de Eaves carga el CNN con strict=False y nombres se_block vs SE_block, así que las capas de atención quedan aleatorias (posible causa de su PCC 0.777). Falta confirmar la ruta ACC2 en Windows. Plugin: plugins/hacnet</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="17">
       <c r="A17" s="27" t="n">
@@ -2938,23 +2974,37 @@
       </c>
       <c r="D17" s="27" t="inlineStr">
         <is>
-          <t>En el repo</t>
+          <t>saved_model/mod_1..10.pickle.dat en el repo (xgboost 1.2.0)</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
-          <t>Docker (MGLTools/MSMS)</t>
-        </is>
-      </c>
-      <c r="F17" s="28" t="n"/>
-      <c r="G17" s="28" t="n"/>
+          <t>Solo Linux: smina (repo), MSMS, MGLTools 1.5.7 (Python 2), AlphaSpace2, xgboost 1.2.0 → en Windows vía Docker/WSL</t>
+        </is>
+      </c>
+      <c r="F17" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H17" s="30" t="n"/>
-      <c r="I17" s="30" t="n"/>
+      <c r="I17" s="30" t="n">
+        <v>0.845</v>
+      </c>
       <c r="J17" s="31">
         <f>IF(AND(ISNUMBER(H17),ISNUMBER(I17)),H17-I17,"")</f>
         <v/>
       </c>
-      <c r="K17" s="28" t="n"/>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: test PASS: 1e66_wat 8.9115 (README 8.893) y 1a30 5.1582. 88 de 92 features de 1a30 iguales a las publicadas por los autores (dataset/test_set.csv); con sus 4 restantes daría 5.1792. pdb_to_xyzr reimplementado en Python (idéntico al de MSMS). Plugin: plugins/delta_linf9_xgb</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="17">
       <c r="A18" s="27" t="n">
@@ -2970,23 +3020,37 @@
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>En el repo</t>
+          <t>model/modelp.pth en el repo + grafos CASF-2016 preparados (release Data, 35 MB)</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
-          <t>Calcular términos Vina</t>
-        </is>
-      </c>
-      <c r="F18" s="28" t="n"/>
-      <c r="G18" s="28" t="n"/>
+          <t>PyTorch 2.2 + DGL 2.2.1 (Python 3.10)</t>
+        </is>
+      </c>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H18" s="30" t="n"/>
-      <c r="I18" s="30" t="n"/>
+      <c r="I18" s="30" t="n">
+        <v>0.831</v>
+      </c>
       <c r="J18" s="31">
         <f>IF(AND(ISNUMBER(H18),ISNUMBER(I18)),H18-I18,"")</f>
         <v/>
       </c>
-      <c r="K18" s="28" t="n"/>
+      <c r="K18" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: NO puede evaluar 1a30: los autores no publican el código que arma grafos y términos Vina, y 1a30 (con 2zcr, 2zy1, 3ag9, 3bv9, 3uri) no está en sus 279 complejos. El test reproduce sus 279 predicciones (dif. máx. 0.00005; PCC 0.810 en esos 279). El código original exige GPU (cuda:0). Ver tarea 6.2. Plugin: plugins/graphscoredta</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="17">
       <c r="A19" s="27" t="n">
@@ -3002,23 +3066,37 @@
       </c>
       <c r="D19" s="27" t="inlineStr">
         <is>
-          <t>En el repo</t>
+          <t>models/saved_model.pth y self-ref_model.pth en el repo</t>
         </is>
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>DGL</t>
-        </is>
-      </c>
-      <c r="F19" s="28" t="n"/>
-      <c r="G19" s="28" t="n"/>
+          <t>PyTorch 2.2 + DGL 2.2.1 + RDKit + Open Babel 3.1.1 + spyrmsd (Python 3.10)</t>
+        </is>
+      </c>
+      <c r="F19" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H19" s="30" t="n"/>
-      <c r="I19" s="30" t="n"/>
+      <c r="I19" s="30" t="n">
+        <v>0.831</v>
+      </c>
       <c r="J19" s="31">
         <f>IF(AND(ISNUMBER(H19),ISNUMBER(I19)),H19-I19,"")</f>
         <v/>
       </c>
-      <c r="K19" s="28" t="n"/>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: test PASS: reproduce el notebook de los autores (1bcu, 10 poses, dif. 3e-6); 1a30 = 5.0653 (modo referencia; self-ref 5.4664). El .sdf de 1a30 no lo lee RDKit: usar .mol2. Eaves usa modo self-ref con saved_model.pth. Plugin: plugins/igmodel</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="17">
       <c r="A20" s="27" t="n">
@@ -3034,23 +3112,37 @@
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>En el repo</t>
+          <t>modelo contrastivo + cabeza de afinidad repeat0 en el repo</t>
         </is>
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>GVP, PyMOL</t>
-        </is>
-      </c>
-      <c r="F20" s="28" t="n"/>
-      <c r="G20" s="28" t="n"/>
+          <t>PyTorch 2.2 + PyG 2.5.3 + torch_scatter/cluster + GVP-GNN + RDKit + PyMOL (Python 3.10)</t>
+        </is>
+      </c>
+      <c r="F20" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H20" s="30" t="n"/>
-      <c r="I20" s="30" t="n"/>
+      <c r="I20" s="30" t="n">
+        <v>0.864</v>
+      </c>
       <c r="J20" s="31">
         <f>IF(AND(ISNUMBER(H20),ISNUMBER(I20)),H20-I20,"")</f>
         <v/>
       </c>
-      <c r="K20" s="28" t="n"/>
+      <c r="K20" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: test PASS: 1bcu del toy set rehecho desde cero = grafos de los autores (4.8575); 1a30 = 5.9318 con ligando sanitizado. Hallazgo: con el .sdf SIN sanitizar (como Eaves) se reproduce exacto su valor 7.7406 → probable causa de su PCC 0.424 (todas sus predicciones altas). Plugin: plugins/conbap</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="17">
       <c r="A21" s="27" t="n">
@@ -3066,23 +3158,37 @@
       </c>
       <c r="D21" s="27" t="inlineStr">
         <is>
-          <t>En el repo</t>
+          <t>result/model.pkl (incompleto)</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>Sin instrucciones de uso</t>
-        </is>
-      </c>
-      <c r="F21" s="28" t="n"/>
-      <c r="G21" s="28" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="H21" s="30" t="n"/>
-      <c r="I21" s="30" t="n"/>
+      <c r="I21" s="30" t="n">
+        <v>0.74</v>
+      </c>
       <c r="J21" s="31">
         <f>IF(AND(ISNUMBER(H21),ISNUMBER(I21)),H21-I21,"")</f>
         <v/>
       </c>
-      <c r="K21" s="28" t="n"/>
+      <c r="K21" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: DESCARTADA. Faltan los modelos word2vec (SMILES 256d y proteína 512d) que usan sus features, y la rama Transformer se crea con pesos aleatorios en cada forward (no está en model.pkl): predicciones no reproducibles. Ver plugins/cpiscore/INSTALL.md</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="17">
       <c r="A22" s="27" t="n">
@@ -3368,7 +3474,7 @@
     <row r="33" ht="15" customHeight="1" s="17">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>Descartadas (sin modelo entrenado): ECIF, MSECIF, Dowker, PerSpect ML, PPS-ML, EISA-Score, GGL-Score, MP-GNN, LGN, FGNN, MFE, MM-DRPNet, DeepTGIN, HaPPy, IMCPiDB-Score, GIaNt, CurvAGN, GCNN01, SMPLIP-Score, aescore.</t>
+          <t>Descartadas (sin modelo entrenado): ECIF, MSECIF, Dowker, PerSpect ML, PPS-ML, EISA-Score, GGL-Score, MP-GNN, LGN, FGNN, MFE, MM-DRPNet, DeepTGIN, HaPPy, IMCPiDB-Score, GIaNt, CurvAGN, GCNN01, SMPLIP-Score, aescore, CPIScore (modelo incompleto, ver nota).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Project sheet: delta_LinF9_XGB passes on Windows (Docker); Docker Desktop installed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J5" s="28" t="inlineStr">
         <is>
-          <t>Miniconda instalado en C:\Users\Admin\miniconda3 (conda 26.9.3, Python 3.14.8, solver libmamba incluido)</t>
+          <t>Miniconda instalado en C:\Users\Admin\miniconda3 (conda 26.9.3, Python 3.14.8, solver libmamba incluido) | 21/10/2026: Docker Desktop 4.96.1 + WSL 2 instalados (necesarios para delta_LinF9_XGB y SF solo-Linux)</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="K17" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: test PASS: 1e66_wat 8.9115 (README 8.893) y 1a30 5.1582. 88 de 92 features de 1a30 iguales a las publicadas por los autores (dataset/test_set.csv); con sus 4 restantes daría 5.1792. pdb_to_xyzr reimplementado en Python (idéntico al de MSMS). Plugin: plugins/delta_linf9_xgb</t>
+          <t>21/10/2026: test PASS: 1e66_wat 8.9115 (README 8.893) y 1a30 5.1582. 88 de 92 features de 1a30 iguales a las publicadas por los autores (dataset/test_set.csv); con sus 4 restantes daría 5.1792. pdb_to_xyzr reimplementado en Python (idéntico al de MSMS). Plugin: plugins/delta_linf9_xgb | 21/10/2026: test PASS en Windows con Docker Desktop 4.96.1 + WSL 2 (demo_delta_linf9_xgb.bat): 1e66_wat 8.9115 y 1a30 5.1582, idénticos a Linux.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Docker test scripts for every plugin (docker_<sf>.bat for Windows, docker_<sf>.sh for Linux) and tools/docker_test_all; tracking sheet: new columns for scripts and Docker/Windows test status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -2322,7 +2322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="16" min="1" max="1"/>
@@ -2335,6 +2335,13 @@
     <col width="12" customWidth="1" style="16" min="8" max="9"/>
     <col width="11" customWidth="1" style="16" min="10" max="10"/>
     <col width="40" customWidth="1" style="16" min="11" max="11"/>
+    <col width="20" customWidth="1" style="17" min="12" max="12"/>
+    <col width="26" customWidth="1" style="17" min="13" max="13"/>
+    <col width="26" customWidth="1" style="17" min="14" max="14"/>
+    <col width="28" customWidth="1" style="17" min="15" max="15"/>
+    <col width="26" customWidth="1" style="17" min="16" max="16"/>
+    <col width="16" customWidth="1" style="17" min="17" max="17"/>
+    <col width="18" customWidth="1" style="17" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="17">
@@ -2347,7 +2354,7 @@
     <row r="2" ht="15" customHeight="1" s="17">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>Completar celdas amarillas. PCC reportado = valor del artículo original en CASF-2016. Diferencia se calcula sola.</t>
+          <t>Completar celdas amarillas. PCC reportado = valor del artículo original en CASF-2016. Diferencia se calcula sola. Columnas L–R: scripts de cada plugin (combi_lab_hub_tmp/plugins/&lt;carpeta&gt;); tools/docker_test_all.bat (.sh) corre todos los tests con Docker y deja un resumen.</t>
         </is>
       </c>
     </row>
@@ -2405,6 +2412,41 @@
       <c r="K4" s="19" t="inlineStr">
         <is>
           <t>Problemas / notas</t>
+        </is>
+      </c>
+      <c r="L4" s="19" t="inlineStr">
+        <is>
+          <t>Plugin (carpeta en plugins/)</t>
+        </is>
+      </c>
+      <c r="M4" s="19" t="inlineStr">
+        <is>
+          <t>Windows conda (.bat)</t>
+        </is>
+      </c>
+      <c r="N4" s="19" t="inlineStr">
+        <is>
+          <t>Imagen Docker</t>
+        </is>
+      </c>
+      <c r="O4" s="19" t="inlineStr">
+        <is>
+          <t>Windows Docker (.bat)</t>
+        </is>
+      </c>
+      <c r="P4" s="19" t="inlineStr">
+        <is>
+          <t>Linux Docker (.sh)</t>
+        </is>
+      </c>
+      <c r="Q4" s="19" t="inlineStr">
+        <is>
+          <t>Test Docker 1a30</t>
+        </is>
+      </c>
+      <c r="R4" s="19" t="inlineStr">
+        <is>
+          <t>Test Windows conda 1a30</t>
         </is>
       </c>
     </row>
@@ -2453,6 +2495,41 @@
           <t>19/10/2026: test 1a30 PASS (pKd 5.6837, igual a los autores). Requiere Python 3.7 + sklearn 0.22.2 exactos; con 0.22.2 los autores reportan PCC 0.793. Plugin: plugins/et_score</t>
         </is>
       </c>
+      <c r="L5" s="28" t="inlineStr">
+        <is>
+          <t>et_score</t>
+        </is>
+      </c>
+      <c r="M5" s="28" t="inlineStr">
+        <is>
+          <t>demo_et_score.bat</t>
+        </is>
+      </c>
+      <c r="N5" s="28" t="inlineStr">
+        <is>
+          <t>combilab/et-score:1.0</t>
+        </is>
+      </c>
+      <c r="O5" s="28" t="inlineStr">
+        <is>
+          <t>docker_et_score.bat</t>
+        </is>
+      </c>
+      <c r="P5" s="28" t="inlineStr">
+        <is>
+          <t>docker_et_score.sh</t>
+        </is>
+      </c>
+      <c r="Q5" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R5" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="17">
       <c r="A6" s="27" t="n">
@@ -2499,6 +2576,41 @@
           <t>19/10/2026: test 1a30 PASS (pKd 5.6171). El repo no trae script de predicción: el modelo usa 104 features filtradas y normalizadas (tabla reconstruida desde total_set_2019.csv). generate_features.py público subcuenta los H de la proteína; corregido leyendo el elemento del PDB. Plugin: plugins/gb_score</t>
         </is>
       </c>
+      <c r="L6" s="28" t="inlineStr">
+        <is>
+          <t>gb_score</t>
+        </is>
+      </c>
+      <c r="M6" s="28" t="inlineStr">
+        <is>
+          <t>demo_gb_score.bat</t>
+        </is>
+      </c>
+      <c r="N6" s="28" t="inlineStr">
+        <is>
+          <t>combilab/gb-score:1.0</t>
+        </is>
+      </c>
+      <c r="O6" s="28" t="inlineStr">
+        <is>
+          <t>docker_gb_score.bat</t>
+        </is>
+      </c>
+      <c r="P6" s="28" t="inlineStr">
+        <is>
+          <t>docker_gb_score.sh</t>
+        </is>
+      </c>
+      <c r="Q6" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R6" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="17">
       <c r="A7" s="27" t="n">
@@ -2545,6 +2657,41 @@
           <t>19/10/2026: test 1a30 PASS. TensorFlow 2.3.4 CPU + sklearn 0.22.1 + Open Babel (ligando .mol2 -&gt; .pdb). Las aguas cristalográficas del PDB cambian la predicción (con aguas 5.4568, CASF sin aguas 5.8866): definir qué archivos usar para el PCC. Eaves et al. reproducen PCC 0.851. Plugin: plugins/onionnet2</t>
         </is>
       </c>
+      <c r="L7" s="28" t="inlineStr">
+        <is>
+          <t>onionnet2</t>
+        </is>
+      </c>
+      <c r="M7" s="28" t="inlineStr">
+        <is>
+          <t>demo_onionnet2.bat</t>
+        </is>
+      </c>
+      <c r="N7" s="28" t="inlineStr">
+        <is>
+          <t>combilab/onionnet2:1.0</t>
+        </is>
+      </c>
+      <c r="O7" s="28" t="inlineStr">
+        <is>
+          <t>docker_onionnet2.bat</t>
+        </is>
+      </c>
+      <c r="P7" s="28" t="inlineStr">
+        <is>
+          <t>docker_onionnet2.sh</t>
+        </is>
+      </c>
+      <c r="Q7" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R7" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="17">
       <c r="A8" s="27" t="n">
@@ -2591,6 +2738,41 @@
           <t>19/10/2026: test 1a30 PASS: pKd 5.4721 idéntico a Sfcnn_2016_test.csv de los autores y 74 poses de docking iguales a test/output2 (dif. máx 0.0007). build_model() carga los pesos desde la carpeta actual. Eaves et al. reproducen PCC 0.789. Plugin: plugins/sfcnn</t>
         </is>
       </c>
+      <c r="L8" s="28" t="inlineStr">
+        <is>
+          <t>sfcnn</t>
+        </is>
+      </c>
+      <c r="M8" s="28" t="inlineStr">
+        <is>
+          <t>demo_sfcnn.bat</t>
+        </is>
+      </c>
+      <c r="N8" s="28" t="inlineStr">
+        <is>
+          <t>combilab/sfcnn:1.0</t>
+        </is>
+      </c>
+      <c r="O8" s="28" t="inlineStr">
+        <is>
+          <t>docker_sfcnn.bat</t>
+        </is>
+      </c>
+      <c r="P8" s="28" t="inlineStr">
+        <is>
+          <t>docker_sfcnn.sh</t>
+        </is>
+      </c>
+      <c r="Q8" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R8" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="17">
       <c r="A9" s="27" t="n">
@@ -2637,6 +2819,41 @@
           <t>19/10/2026: test 1a30 PASS (5.8930 con core.tar.bz2 de los autores; 5.6216 con CASF .mol2). El .sdf de CASF de 1a30 no lo lee RDKit: usar core.tar.bz2 de los autores. demo/result.csv es de 2022 (modelo viejo), no sirve de referencia. Plugin: plugins/planet</t>
         </is>
       </c>
+      <c r="L9" s="28" t="inlineStr">
+        <is>
+          <t>planet</t>
+        </is>
+      </c>
+      <c r="M9" s="28" t="inlineStr">
+        <is>
+          <t>demo_planet.bat</t>
+        </is>
+      </c>
+      <c r="N9" s="28" t="inlineStr">
+        <is>
+          <t>combilab/planet:1.0</t>
+        </is>
+      </c>
+      <c r="O9" s="28" t="inlineStr">
+        <is>
+          <t>docker_planet.bat</t>
+        </is>
+      </c>
+      <c r="P9" s="28" t="inlineStr">
+        <is>
+          <t>docker_planet.sh</t>
+        </is>
+      </c>
+      <c r="Q9" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R9" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="17">
       <c r="A10" s="27" t="n">
@@ -2683,6 +2900,41 @@
           <t>20/10/2026: test 1a30 PASS (pKd 5.1040 con pocket, idéntico a Eaves et al.; 6.5326 con proteína completa). Usar _pocket.pdb: con la proteína completa Eaves obtiene PCC 0.071, con el pocket 0.669 (no reproduce el 0.86 del artículo). Ligando como SMILES desde el .mol2. El checkpoint es un modelo pickleado con clases __main__.*: el wrapper las redirige. Plugin: plugins/eggnn</t>
         </is>
       </c>
+      <c r="L10" s="28" t="inlineStr">
+        <is>
+          <t>eggnn</t>
+        </is>
+      </c>
+      <c r="M10" s="28" t="inlineStr">
+        <is>
+          <t>demo_eggnn.bat</t>
+        </is>
+      </c>
+      <c r="N10" s="28" t="inlineStr">
+        <is>
+          <t>combilab/eggnn:1.0</t>
+        </is>
+      </c>
+      <c r="O10" s="28" t="inlineStr">
+        <is>
+          <t>docker_eggnn.bat</t>
+        </is>
+      </c>
+      <c r="P10" s="28" t="inlineStr">
+        <is>
+          <t>docker_eggnn.sh</t>
+        </is>
+      </c>
+      <c r="Q10" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R10" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="17">
       <c r="A11" s="27" t="n">
@@ -2729,6 +2981,41 @@
           <t>20/10/2026: test 1a30 PASS (modelos 4.3883 / 6.3427 / 6.4380, media 5.7230, igual a los scripts de los autores). Nuestro grafo de 1a30 es idéntico al preparado por los autores (Zenodo 7490623); con sus 285 grafos del core set: PCC 0.844 / 0.843 / 0.832, 0.855 con la media. Pocket con PyMOL a 5 Å + obabel -d. Eaves et al. reproducen PCC 0.85. Plugin: plugins/gign</t>
         </is>
       </c>
+      <c r="L11" s="28" t="inlineStr">
+        <is>
+          <t>gign</t>
+        </is>
+      </c>
+      <c r="M11" s="28" t="inlineStr">
+        <is>
+          <t>demo_gign.bat</t>
+        </is>
+      </c>
+      <c r="N11" s="28" t="inlineStr">
+        <is>
+          <t>combilab/gign:1.0</t>
+        </is>
+      </c>
+      <c r="O11" s="28" t="inlineStr">
+        <is>
+          <t>docker_gign.bat</t>
+        </is>
+      </c>
+      <c r="P11" s="28" t="inlineStr">
+        <is>
+          <t>docker_gign.sh</t>
+        </is>
+      </c>
+      <c r="Q11" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R11" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="17">
       <c r="A12" s="27" t="n">
@@ -2775,6 +3062,41 @@
           <t>20/10/2026: test 1a30 PASS (5.5024 / 5.8087 / 5.0898, media 5.4670, igual a los scripts de los autores). Código para DGL 0.9: copy_src mapeado a copy_u; el modelo modifica el grafo, se recarga por modelo. Falta calcular el PCC del core set. Eaves et al. reproducen PCC 0.851. Plugin: plugins/ehign_pla</t>
         </is>
       </c>
+      <c r="L12" s="28" t="inlineStr">
+        <is>
+          <t>ehign_pla</t>
+        </is>
+      </c>
+      <c r="M12" s="28" t="inlineStr">
+        <is>
+          <t>demo_ehign_pla.bat</t>
+        </is>
+      </c>
+      <c r="N12" s="28" t="inlineStr">
+        <is>
+          <t>combilab/ehign_pla:1.0</t>
+        </is>
+      </c>
+      <c r="O12" s="28" t="inlineStr">
+        <is>
+          <t>docker_ehign_pla.bat</t>
+        </is>
+      </c>
+      <c r="P12" s="28" t="inlineStr">
+        <is>
+          <t>docker_ehign_pla.sh</t>
+        </is>
+      </c>
+      <c r="Q12" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R12" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="17">
       <c r="A13" s="27" t="n">
@@ -2821,6 +3143,41 @@
           <t>20/10/2026: test 1a30 PASS (pKd 5.0950, idéntico a Eaves et al.; 3jvr 4.7484 y features iguales a los de los autores). No requiere HTMD (htmd 2.0.6 pide acemd3 no público): se usa moleculekit 1.11.5 con la preparación corregida de Eaves, sin el fallback HTMD/CHARMM. Checkpoint guardado en GPU, se carga en CPU. Eaves et al. reproducen PCC 0.862. Plugin: plugins/sacnn</t>
         </is>
       </c>
+      <c r="L13" s="28" t="inlineStr">
+        <is>
+          <t>sacnn</t>
+        </is>
+      </c>
+      <c r="M13" s="28" t="inlineStr">
+        <is>
+          <t>demo_sacnn.bat</t>
+        </is>
+      </c>
+      <c r="N13" s="28" t="inlineStr">
+        <is>
+          <t>combilab/sacnn:1.0</t>
+        </is>
+      </c>
+      <c r="O13" s="28" t="inlineStr">
+        <is>
+          <t>docker_sacnn.bat</t>
+        </is>
+      </c>
+      <c r="P13" s="28" t="inlineStr">
+        <is>
+          <t>docker_sacnn.sh</t>
+        </is>
+      </c>
+      <c r="Q13" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R13" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="17">
       <c r="A14" s="27" t="n">
@@ -2867,6 +3224,41 @@
           <t>20/10/2026: test 1a30 PASS (6.3185 con los datos preprocesados de los autores, igual a su kfold_result.csv; 6.2026 con archivos CASF: mismo SMILES y secuencia, pocket CASF 51 vs 56 residuos). Con los datos de los autores reproduce su kfold_result.csv en 278 complejos (PCC 0.853). Los pocket de CASF no tienen cadena: el wrapper asigna cada residuo por número y nombre en orden (A y luego B). Eaves et al. reproducen PCC 0.819. Plugin: plugins/deattentiondta</t>
         </is>
       </c>
+      <c r="L14" s="28" t="inlineStr">
+        <is>
+          <t>deattentiondta</t>
+        </is>
+      </c>
+      <c r="M14" s="28" t="inlineStr">
+        <is>
+          <t>demo_deattentiondta.bat</t>
+        </is>
+      </c>
+      <c r="N14" s="28" t="inlineStr">
+        <is>
+          <t>combilab/deattentiondta:1.0</t>
+        </is>
+      </c>
+      <c r="O14" s="28" t="inlineStr">
+        <is>
+          <t>docker_deattentiondta.bat</t>
+        </is>
+      </c>
+      <c r="P14" s="28" t="inlineStr">
+        <is>
+          <t>docker_deattentiondta.sh</t>
+        </is>
+      </c>
+      <c r="Q14" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R14" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="17">
       <c r="A15" s="27" t="n">
@@ -2913,6 +3305,41 @@
           <t>21/10/2026: test 1a30 PASS (pKd 4.4640, valor propio). El modelo es una red PyG 1.4 pickleada: su GCNConv normaliza por el grado del nodo origen (PyG actual: destino) y el grafo del pocket es dirigido; con la capa actual 1a30 da 6.4782. Se usa una copia exacta de la capa vieja. Plugin: plugins/deepbindgcn</t>
         </is>
       </c>
+      <c r="L15" s="28" t="inlineStr">
+        <is>
+          <t>deepbindgcn</t>
+        </is>
+      </c>
+      <c r="M15" s="28" t="inlineStr">
+        <is>
+          <t>demo_deepbindgcn.bat</t>
+        </is>
+      </c>
+      <c r="N15" s="28" t="inlineStr">
+        <is>
+          <t>combilab/deepbindgcn:1.0</t>
+        </is>
+      </c>
+      <c r="O15" s="28" t="inlineStr">
+        <is>
+          <t>docker_deepbindgcn.bat</t>
+        </is>
+      </c>
+      <c r="P15" s="28" t="inlineStr">
+        <is>
+          <t>docker_deepbindgcn.sh</t>
+        </is>
+      </c>
+      <c r="Q15" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R15" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="17">
       <c r="A16" s="27" t="n">
@@ -2959,6 +3386,41 @@
           <t>21/10/2026: test 1a30 PASS con ChargeFW2 3.0.0 (pKd 4.9114, valor propio). El servidor de cargas original ya no existe: se usa ACC2 (internet) o ChargeFW2 compilado en Docker. Hallazgo: el notebook/fork de Eaves carga el CNN con strict=False y nombres se_block vs SE_block, así que las capas de atención quedan aleatorias (posible causa de su PCC 0.777). Plugin: plugins/hacnet | 21/10/2026: test 1a30 PASS en Windows (demo_hacnet.bat). Arreglos: entorno con glib de conda-forge (libglib 2.88.3 del canal defaults pisaba intl-8.dll; fix_env_hacnet.bat) y cargas por la API de Atomic Charge Calculator III (acc.biodata.ceitec.cz; la URL de ACC2 da 405).</t>
         </is>
       </c>
+      <c r="L16" s="28" t="inlineStr">
+        <is>
+          <t>hacnet</t>
+        </is>
+      </c>
+      <c r="M16" s="28" t="inlineStr">
+        <is>
+          <t>demo_hacnet.bat</t>
+        </is>
+      </c>
+      <c r="N16" s="28" t="inlineStr">
+        <is>
+          <t>combilab/hacnet:1.0</t>
+        </is>
+      </c>
+      <c r="O16" s="28" t="inlineStr">
+        <is>
+          <t>docker_hacnet.bat</t>
+        </is>
+      </c>
+      <c r="P16" s="28" t="inlineStr">
+        <is>
+          <t>docker_hacnet.sh</t>
+        </is>
+      </c>
+      <c r="Q16" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R16" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="17">
       <c r="A17" s="27" t="n">
@@ -3005,6 +3467,41 @@
           <t>21/10/2026: test PASS: 1e66_wat 8.9115 (README 8.893) y 1a30 5.1582. 88 de 92 features de 1a30 iguales a las publicadas por los autores (dataset/test_set.csv); con sus 4 restantes daría 5.1792. pdb_to_xyzr reimplementado en Python (idéntico al de MSMS). Plugin: plugins/delta_linf9_xgb | 21/10/2026: test PASS en Windows con Docker Desktop 4.96.1 + WSL 2 (demo_delta_linf9_xgb.bat): 1e66_wat 8.9115 y 1a30 5.1582, idénticos a Linux.</t>
         </is>
       </c>
+      <c r="L17" s="28" t="inlineStr">
+        <is>
+          <t>delta_linf9_xgb</t>
+        </is>
+      </c>
+      <c r="M17" s="28" t="inlineStr">
+        <is>
+          <t>no (solo Linux) → usar Docker</t>
+        </is>
+      </c>
+      <c r="N17" s="28" t="inlineStr">
+        <is>
+          <t>combilab/delta_linf9_xgb:1.0</t>
+        </is>
+      </c>
+      <c r="O17" s="28" t="inlineStr">
+        <is>
+          <t>docker_delta_linf9_xgb.bat</t>
+        </is>
+      </c>
+      <c r="P17" s="28" t="inlineStr">
+        <is>
+          <t>docker_delta_linf9_xgb.sh</t>
+        </is>
+      </c>
+      <c r="Q17" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R17" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="17">
       <c r="A18" s="27" t="n">
@@ -3051,6 +3548,41 @@
           <t>21/10/2026: NO puede evaluar 1a30: los autores no publican el código que arma grafos y términos Vina, y 1a30 (con 2zcr, 2zy1, 3ag9, 3bv9, 3uri) no está en sus 279 complejos. El test reproduce sus 279 predicciones (dif. máx. 0.00005; PCC 0.810 en esos 279). El código original exige GPU (cuda:0). Ver tarea 6.2. Plugin: plugins/graphscoredta</t>
         </is>
       </c>
+      <c r="L18" s="28" t="inlineStr">
+        <is>
+          <t>graphscoredta</t>
+        </is>
+      </c>
+      <c r="M18" s="28" t="inlineStr">
+        <is>
+          <t>demo_graphscoredta.bat</t>
+        </is>
+      </c>
+      <c r="N18" s="28" t="inlineStr">
+        <is>
+          <t>combilab/graphscoredta:1.0</t>
+        </is>
+      </c>
+      <c r="O18" s="28" t="inlineStr">
+        <is>
+          <t>docker_graphscoredta.bat</t>
+        </is>
+      </c>
+      <c r="P18" s="28" t="inlineStr">
+        <is>
+          <t>docker_graphscoredta.sh</t>
+        </is>
+      </c>
+      <c r="Q18" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R18" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="17">
       <c r="A19" s="27" t="n">
@@ -3097,6 +3629,41 @@
           <t>21/10/2026: test PASS: reproduce el notebook de los autores (1bcu, 10 poses, dif. 3e-6); 1a30 = 5.0653 (modo referencia; self-ref 5.4664). El .sdf de 1a30 no lo lee RDKit: usar .mol2. Eaves usa modo self-ref con saved_model.pth. Plugin: plugins/igmodel</t>
         </is>
       </c>
+      <c r="L19" s="28" t="inlineStr">
+        <is>
+          <t>igmodel</t>
+        </is>
+      </c>
+      <c r="M19" s="28" t="inlineStr">
+        <is>
+          <t>demo_igmodel.bat</t>
+        </is>
+      </c>
+      <c r="N19" s="28" t="inlineStr">
+        <is>
+          <t>combilab/igmodel:1.0</t>
+        </is>
+      </c>
+      <c r="O19" s="28" t="inlineStr">
+        <is>
+          <t>docker_igmodel.bat</t>
+        </is>
+      </c>
+      <c r="P19" s="28" t="inlineStr">
+        <is>
+          <t>docker_igmodel.sh</t>
+        </is>
+      </c>
+      <c r="Q19" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R19" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="17">
       <c r="A20" s="27" t="n">
@@ -3143,6 +3710,41 @@
           <t>21/10/2026: test PASS: 1bcu del toy set rehecho desde cero = grafos de los autores (4.8575); 1a30 = 5.9318 con ligando sanitizado. Hallazgo: con el .sdf SIN sanitizar (como Eaves) se reproduce exacto su valor 7.7406 → probable causa de su PCC 0.424 (todas sus predicciones altas). Plugin: plugins/conbap</t>
         </is>
       </c>
+      <c r="L20" s="28" t="inlineStr">
+        <is>
+          <t>conbap</t>
+        </is>
+      </c>
+      <c r="M20" s="28" t="inlineStr">
+        <is>
+          <t>demo_conbap.bat</t>
+        </is>
+      </c>
+      <c r="N20" s="28" t="inlineStr">
+        <is>
+          <t>combilab/conbap:1.0</t>
+        </is>
+      </c>
+      <c r="O20" s="28" t="inlineStr">
+        <is>
+          <t>docker_conbap.bat</t>
+        </is>
+      </c>
+      <c r="P20" s="28" t="inlineStr">
+        <is>
+          <t>docker_conbap.sh</t>
+        </is>
+      </c>
+      <c r="Q20" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R20" s="30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="17">
       <c r="A21" s="27" t="n">
@@ -3187,6 +3789,41 @@
       <c r="K21" s="28" t="inlineStr">
         <is>
           <t>21/10/2026: DESCARTADA. Faltan los modelos word2vec (SMILES 256d y proteína 512d) que usan sus features, y la rama Transformer se crea con pesos aleatorios en cada forward (no está en model.pkl): predicciones no reproducibles. Ver plugins/cpiscore/INSTALL.md</t>
+        </is>
+      </c>
+      <c r="L21" s="28" t="inlineStr">
+        <is>
+          <t>cpiscore</t>
+        </is>
+      </c>
+      <c r="M21" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N21" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O21" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P21" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q21" s="30" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="R21" s="30" t="inlineStr">
+        <is>
+          <t>No aplica</t>
         </is>
       </c>
     </row>
@@ -3491,10 +4128,13 @@
       <formula>"Parcial"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="F5:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Sí,No,Parcial"</formula1>
       <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation sqref="Q5:R31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,PASS,FAIL,No aplica"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Add RFL-Score plugin (Level 1): R model test on Windows, full 160-feature pipeline with Docker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -628,19 +628,19 @@
         </is>
       </c>
       <c r="B4" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A4)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A4)</f>
         <v/>
       </c>
       <c r="C4" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A4,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A4,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D4" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A4,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A4,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E4" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A4,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A4,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F4" s="21">
@@ -655,19 +655,19 @@
         </is>
       </c>
       <c r="B5" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A5)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A5)</f>
         <v/>
       </c>
       <c r="C5" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A5,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A5,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D5" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A5,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A5,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E5" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A5,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A5,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F5" s="21">
@@ -682,19 +682,19 @@
         </is>
       </c>
       <c r="B6" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A6)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A6)</f>
         <v/>
       </c>
       <c r="C6" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A6,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A6,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D6" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A6,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A6,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E6" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A6,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A6,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F6" s="21">
@@ -709,19 +709,19 @@
         </is>
       </c>
       <c r="B7" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A7)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A7)</f>
         <v/>
       </c>
       <c r="C7" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A7,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A7,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D7" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A7,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A7,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E7" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A7,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A7,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F7" s="21">
@@ -736,19 +736,19 @@
         </is>
       </c>
       <c r="B8" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A8)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A8)</f>
         <v/>
       </c>
       <c r="C8" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A8,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A8,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D8" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A8,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A8,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E8" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A8,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A8,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F8" s="21">
@@ -763,19 +763,19 @@
         </is>
       </c>
       <c r="B9" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A9)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A9)</f>
         <v/>
       </c>
       <c r="C9" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A9,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A9,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D9" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A9,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A9,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E9" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A9,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A9,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F9" s="21">
@@ -790,19 +790,19 @@
         </is>
       </c>
       <c r="B10" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A10)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A10)</f>
         <v/>
       </c>
       <c r="C10" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A10,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A10,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D10" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A10,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A10,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E10" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A10,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A10,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F10" s="21">
@@ -817,19 +817,19 @@
         </is>
       </c>
       <c r="B11" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A11)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A11)</f>
         <v/>
       </c>
       <c r="C11" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A11,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A11,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D11" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A11,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A11,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E11" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A11,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A11,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F11" s="21">
@@ -844,19 +844,19 @@
         </is>
       </c>
       <c r="B12" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A12)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A12)</f>
         <v/>
       </c>
       <c r="C12" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A12,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A12,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D12" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A12,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A12,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E12" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A12,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A12,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F12" s="21">
@@ -871,19 +871,19 @@
         </is>
       </c>
       <c r="B13" s="20">
-        <f>COUNTIF(Etapas!$B$5:$B$34,A13)</f>
+        <f>COUNTIF(Etapas!$B$5:$B$40,A13)</f>
         <v/>
       </c>
       <c r="C13" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A13,Etapas!$F$5:$F$34,"Completada")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A13,Etapas!$F$5:$F$40,"Completada")</f>
         <v/>
       </c>
       <c r="D13" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A13,Etapas!$F$5:$F$34,"En progreso")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A13,Etapas!$F$5:$F$40,"En progreso")</f>
         <v/>
       </c>
       <c r="E13" s="20">
-        <f>COUNTIFS(Etapas!$B$5:$B$34,A13,Etapas!$F$5:$F$34,"Pendiente")</f>
+        <f>COUNTIFS(Etapas!$B$5:$B$40,A13,Etapas!$F$5:$F$40,"Pendiente")</f>
         <v/>
       </c>
       <c r="F13" s="21">
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="16" min="1" max="1"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>Nivel 1 (10), Nivel 2 (7), Nivel 3 (10), descartadas (20, sin modelo entrenado)</t>
+          <t>Nivel 1 (11), Nivel 2 (7), Nivel 3 (9), descartadas (20, sin modelo entrenado)</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
@@ -1568,7 +1568,11 @@
       <c r="G16" s="28" t="n"/>
       <c r="H16" s="29" t="n"/>
       <c r="I16" s="29" t="n"/>
-      <c r="J16" s="28" t="n"/>
+      <c r="J16" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | 21/10/2026: RFL-Score pasa del Nivel 3 al Nivel 1</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="26.25" customHeight="1" s="17">
       <c r="A17" s="27" t="inlineStr">
@@ -2122,7 +2126,7 @@
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>PointNet, PIGNet2, Dynaformer, TopoFormer, BAPA, CGraphDTA, EGNA, HydraScreen, RFL-Score, P3-Score</t>
+          <t>PointNet, PIGNet2, Dynaformer, TopoFormer, BAPA, CGraphDTA, EGNA, HydraScreen, P3-Score</t>
         </is>
       </c>
       <c r="E30" s="27" t="inlineStr">
@@ -2287,6 +2291,50 @@
       <c r="H34" s="29" t="n"/>
       <c r="I34" s="29" t="n"/>
       <c r="J34" s="28" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>5. Pruebas Nivel 1 (CPU, modelo listo)</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>RFL-Score (SF de combi-lab)</t>
+        </is>
+      </c>
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>Plugin plugins/rfl_score: test liviano con R en Windows + pipeline completo de 160 features con Docker</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F35" s="28" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n"/>
+      <c r="H35" s="29" t="n">
+        <v>46316</v>
+      </c>
+      <c r="I35" s="29" t="n">
+        <v>46316</v>
+      </c>
+      <c r="J35" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: test 1a30 PASS en Linux: modelo 4.4494 con las features de los autores; pipeline completo = mismas 160 features y 4.4494. Falta confirmar demo_rfl_score.bat (Windows conda) y docker_rfl_score.bat en la PC del laboratorio. El core set entra en run_coreset_level1.bat (vía Docker) para el video (8.1)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:J33"/>
@@ -2305,7 +2353,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="F5:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Pendiente,En progreso,Completada,Bloqueada"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3262,24 +3310,24 @@
     </row>
     <row r="15" ht="15" customHeight="1" s="17">
       <c r="A15" s="27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" s="27" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>DeepBindGCN</t>
+          <t>RFL-Score</t>
         </is>
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>GitHub release v1.0.0: full_model_out2000_RG.model (MD5 aaa69454…)</t>
+          <t>scoring/RScript/model/scoring_function_160.rda en el repo (Random Forest de R, 160 features; MD5 d1ad344e…)</t>
         </is>
       </c>
       <c r="E15" s="27" t="inlineStr">
         <is>
-          <t>PyTorch 2.2 + PyG 2.5.3 + RDKit (Python 3.10)</t>
+          <t>R + randomForest (test Windows conda). Pipeline completo de features (solo Linux → Docker): Open Babel 2.4.1, PaDEL (Java 11), DSSP, MGLTools 1.5.7, vina4dv, ODDT 0.7, RDKit 2020.09 (Python 3.7)</t>
         </is>
       </c>
       <c r="F15" s="28" t="inlineStr">
@@ -3293,41 +3341,39 @@
         </is>
       </c>
       <c r="H15" s="30" t="n"/>
-      <c r="I15" s="30" t="n">
-        <v>0.75</v>
-      </c>
+      <c r="I15" s="30" t="n"/>
       <c r="J15" s="31">
         <f>IF(AND(ISNUMBER(H15),ISNUMBER(I15)),H15-I15,"")</f>
         <v/>
       </c>
       <c r="K15" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: test 1a30 PASS (pKd 4.4640, valor propio). El modelo es una red PyG 1.4 pickleada: su GCNConv normaliza por el grado del nodo origen (PyG actual: destino) y el grafo del pocket es dirigido; con la capa actual 1a30 da 6.4782. Se usa una copia exacta de la capa vieja. Plugin: plugins/deepbindgcn</t>
+          <t>21/10/2026: SF propia de combi-lab (Arrua et al., IEEE CIBCB 2024). Test 1a30 PASS: el modelo con las 160 features de los autores (examples/1a30/1a30_160_input.csv) da 4.4494; el pipeline completo desde los archivos de CASF reproduce las 160 features EXACTAS (0 diferencias) y el mismo 4.4494. Con examples/all_160_input.csv da 4.5071 (otra versión de los descriptores RDKit 3D). Adaptaciones sin cambiar el código: wrapper de dssp para DSSP 4.2 (ya no acepta -i/-o) y prepare_ligand4.py corrido desde la carpeta del ligando. La secuencia FASTA se baja de RCSB (como los autores; incluye la cadena del péptido inhibidor); armada desde el PDB 1a30 da 4.4739. Completar PCC reportado. El RFL-Score.zip de la tabla es una versión anterior (2022), sirve para el test liviano; Docker usa el commit 2020d90. Plugin: plugins/rfl_score</t>
         </is>
       </c>
       <c r="L15" s="28" t="inlineStr">
         <is>
-          <t>deepbindgcn</t>
+          <t>rfl_score</t>
         </is>
       </c>
       <c r="M15" s="28" t="inlineStr">
         <is>
-          <t>demo_deepbindgcn.bat</t>
+          <t>demo_rfl_score.bat (solo modelo)</t>
         </is>
       </c>
       <c r="N15" s="28" t="inlineStr">
         <is>
-          <t>combilab/deepbindgcn:1.0</t>
+          <t>combilab/rfl_score:1.0</t>
         </is>
       </c>
       <c r="O15" s="28" t="inlineStr">
         <is>
-          <t>docker_deepbindgcn.bat</t>
+          <t>docker_rfl_score.bat</t>
         </is>
       </c>
       <c r="P15" s="28" t="inlineStr">
         <is>
-          <t>docker_deepbindgcn.sh</t>
+          <t>docker_rfl_score.sh</t>
         </is>
       </c>
       <c r="Q15" s="30" t="inlineStr">
@@ -3346,21 +3392,21 @@
         <v>2</v>
       </c>
       <c r="B16" s="27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>HAC-Net</t>
+          <t>DeepBindGCN</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>HACNet/parameter_files en el repo (4 .pt) + paquete PyPI HACNet 1.4.3</t>
+          <t>GitHub release v1.0.0: full_model_out2000_RG.model (MD5 aaa69454…)</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
         <is>
-          <t>PyTorch 2.2 + PyG 2.5.3 + Open Babel + PyMOL; cargas EqEq: servicio web ACC2 o ChargeFW2 local (Docker)</t>
+          <t>PyTorch 2.2 + PyG 2.5.3 + RDKit (Python 3.10)</t>
         </is>
       </c>
       <c r="F16" s="28" t="inlineStr">
@@ -3375,7 +3421,7 @@
       </c>
       <c r="H16" s="30" t="n"/>
       <c r="I16" s="30" t="n">
-        <v>0.846</v>
+        <v>0.75</v>
       </c>
       <c r="J16" s="31">
         <f>IF(AND(ISNUMBER(H16),ISNUMBER(I16)),H16-I16,"")</f>
@@ -3383,32 +3429,32 @@
       </c>
       <c r="K16" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: test 1a30 PASS con ChargeFW2 3.0.0 (pKd 4.9114, valor propio). El servidor de cargas original ya no existe: se usa ACC2 (internet) o ChargeFW2 compilado en Docker. Hallazgo: el notebook/fork de Eaves carga el CNN con strict=False y nombres se_block vs SE_block, así que las capas de atención quedan aleatorias (posible causa de su PCC 0.777). Plugin: plugins/hacnet | 21/10/2026: test 1a30 PASS en Windows (demo_hacnet.bat). Arreglos: entorno con glib de conda-forge (libglib 2.88.3 del canal defaults pisaba intl-8.dll; fix_env_hacnet.bat) y cargas por la API de Atomic Charge Calculator III (acc.biodata.ceitec.cz; la URL de ACC2 da 405).</t>
+          <t>21/10/2026: test 1a30 PASS (pKd 4.4640, valor propio). El modelo es una red PyG 1.4 pickleada: su GCNConv normaliza por el grado del nodo origen (PyG actual: destino) y el grafo del pocket es dirigido; con la capa actual 1a30 da 6.4782. Se usa una copia exacta de la capa vieja. Plugin: plugins/deepbindgcn</t>
         </is>
       </c>
       <c r="L16" s="28" t="inlineStr">
         <is>
-          <t>hacnet</t>
+          <t>deepbindgcn</t>
         </is>
       </c>
       <c r="M16" s="28" t="inlineStr">
         <is>
-          <t>demo_hacnet.bat</t>
+          <t>demo_deepbindgcn.bat</t>
         </is>
       </c>
       <c r="N16" s="28" t="inlineStr">
         <is>
-          <t>combilab/hacnet:1.0</t>
+          <t>combilab/deepbindgcn:1.0</t>
         </is>
       </c>
       <c r="O16" s="28" t="inlineStr">
         <is>
-          <t>docker_hacnet.bat</t>
+          <t>docker_deepbindgcn.bat</t>
         </is>
       </c>
       <c r="P16" s="28" t="inlineStr">
         <is>
-          <t>docker_hacnet.sh</t>
+          <t>docker_deepbindgcn.sh</t>
         </is>
       </c>
       <c r="Q16" s="30" t="inlineStr">
@@ -3418,7 +3464,7 @@
       </c>
       <c r="R16" s="30" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -3427,21 +3473,21 @@
         <v>2</v>
       </c>
       <c r="B17" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>delta_LinF9_XGB</t>
+          <t>HAC-Net</t>
         </is>
       </c>
       <c r="D17" s="27" t="inlineStr">
         <is>
-          <t>saved_model/mod_1..10.pickle.dat en el repo (xgboost 1.2.0)</t>
+          <t>HACNet/parameter_files en el repo (4 .pt) + paquete PyPI HACNet 1.4.3</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
-          <t>Solo Linux: smina (repo), MSMS, MGLTools 1.5.7 (Python 2), AlphaSpace2, xgboost 1.2.0 → en Windows vía Docker/WSL</t>
+          <t>PyTorch 2.2 + PyG 2.5.3 + Open Babel + PyMOL; cargas EqEq: servicio web ACC2 o ChargeFW2 local (Docker)</t>
         </is>
       </c>
       <c r="F17" s="28" t="inlineStr">
@@ -3456,7 +3502,7 @@
       </c>
       <c r="H17" s="30" t="n"/>
       <c r="I17" s="30" t="n">
-        <v>0.845</v>
+        <v>0.846</v>
       </c>
       <c r="J17" s="31">
         <f>IF(AND(ISNUMBER(H17),ISNUMBER(I17)),H17-I17,"")</f>
@@ -3464,42 +3510,42 @@
       </c>
       <c r="K17" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: test PASS: 1e66_wat 8.9115 (README 8.893) y 1a30 5.1582. 88 de 92 features de 1a30 iguales a las publicadas por los autores (dataset/test_set.csv); con sus 4 restantes daría 5.1792. pdb_to_xyzr reimplementado en Python (idéntico al de MSMS). Plugin: plugins/delta_linf9_xgb | 21/10/2026: test PASS en Windows con Docker Desktop 4.96.1 + WSL 2 (demo_delta_linf9_xgb.bat): 1e66_wat 8.9115 y 1a30 5.1582, idénticos a Linux.</t>
+          <t>21/10/2026: test 1a30 PASS con ChargeFW2 3.0.0 (pKd 4.9114, valor propio). El servidor de cargas original ya no existe: se usa ACC2 (internet) o ChargeFW2 compilado en Docker. Hallazgo: el notebook/fork de Eaves carga el CNN con strict=False y nombres se_block vs SE_block, así que las capas de atención quedan aleatorias (posible causa de su PCC 0.777). Plugin: plugins/hacnet | 21/10/2026: test 1a30 PASS en Windows (demo_hacnet.bat). Arreglos: entorno con glib de conda-forge (libglib 2.88.3 del canal defaults pisaba intl-8.dll; fix_env_hacnet.bat) y cargas por la API de Atomic Charge Calculator III (acc.biodata.ceitec.cz; la URL de ACC2 da 405).</t>
         </is>
       </c>
       <c r="L17" s="28" t="inlineStr">
         <is>
-          <t>delta_linf9_xgb</t>
+          <t>hacnet</t>
         </is>
       </c>
       <c r="M17" s="28" t="inlineStr">
         <is>
-          <t>no (solo Linux) → usar Docker</t>
+          <t>demo_hacnet.bat</t>
         </is>
       </c>
       <c r="N17" s="28" t="inlineStr">
         <is>
-          <t>combilab/delta_linf9_xgb:1.0</t>
+          <t>combilab/hacnet:1.0</t>
         </is>
       </c>
       <c r="O17" s="28" t="inlineStr">
         <is>
-          <t>docker_delta_linf9_xgb.bat</t>
+          <t>docker_hacnet.bat</t>
         </is>
       </c>
       <c r="P17" s="28" t="inlineStr">
         <is>
-          <t>docker_delta_linf9_xgb.sh</t>
+          <t>docker_hacnet.sh</t>
         </is>
       </c>
       <c r="Q17" s="30" t="inlineStr">
         <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R17" s="30" t="inlineStr">
+        <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="R17" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
@@ -3508,21 +3554,21 @@
         <v>2</v>
       </c>
       <c r="B18" s="27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>GraphscoreDTA</t>
+          <t>delta_LinF9_XGB</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>model/modelp.pth en el repo + grafos CASF-2016 preparados (release Data, 35 MB)</t>
+          <t>saved_model/mod_1..10.pickle.dat en el repo (xgboost 1.2.0)</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
-          <t>PyTorch 2.2 + DGL 2.2.1 (Python 3.10)</t>
+          <t>Solo Linux: smina (repo), MSMS, MGLTools 1.5.7 (Python 2), AlphaSpace2, xgboost 1.2.0 → en Windows vía Docker/WSL</t>
         </is>
       </c>
       <c r="F18" s="28" t="inlineStr">
@@ -3537,7 +3583,7 @@
       </c>
       <c r="H18" s="30" t="n"/>
       <c r="I18" s="30" t="n">
-        <v>0.831</v>
+        <v>0.845</v>
       </c>
       <c r="J18" s="31">
         <f>IF(AND(ISNUMBER(H18),ISNUMBER(I18)),H18-I18,"")</f>
@@ -3545,42 +3591,42 @@
       </c>
       <c r="K18" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: NO puede evaluar 1a30: los autores no publican el código que arma grafos y términos Vina, y 1a30 (con 2zcr, 2zy1, 3ag9, 3bv9, 3uri) no está en sus 279 complejos. El test reproduce sus 279 predicciones (dif. máx. 0.00005; PCC 0.810 en esos 279). El código original exige GPU (cuda:0). Ver tarea 6.2. Plugin: plugins/graphscoredta</t>
+          <t>21/10/2026: test PASS: 1e66_wat 8.9115 (README 8.893) y 1a30 5.1582. 88 de 92 features de 1a30 iguales a las publicadas por los autores (dataset/test_set.csv); con sus 4 restantes daría 5.1792. pdb_to_xyzr reimplementado en Python (idéntico al de MSMS). Plugin: plugins/delta_linf9_xgb | 21/10/2026: test PASS en Windows con Docker Desktop 4.96.1 + WSL 2 (demo_delta_linf9_xgb.bat): 1e66_wat 8.9115 y 1a30 5.1582, idénticos a Linux.</t>
         </is>
       </c>
       <c r="L18" s="28" t="inlineStr">
         <is>
-          <t>graphscoredta</t>
+          <t>delta_linf9_xgb</t>
         </is>
       </c>
       <c r="M18" s="28" t="inlineStr">
         <is>
-          <t>demo_graphscoredta.bat</t>
+          <t>no (solo Linux) → usar Docker</t>
         </is>
       </c>
       <c r="N18" s="28" t="inlineStr">
         <is>
-          <t>combilab/graphscoredta:1.0</t>
+          <t>combilab/delta_linf9_xgb:1.0</t>
         </is>
       </c>
       <c r="O18" s="28" t="inlineStr">
         <is>
-          <t>docker_graphscoredta.bat</t>
+          <t>docker_delta_linf9_xgb.bat</t>
         </is>
       </c>
       <c r="P18" s="28" t="inlineStr">
         <is>
-          <t>docker_graphscoredta.sh</t>
+          <t>docker_delta_linf9_xgb.sh</t>
         </is>
       </c>
       <c r="Q18" s="30" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R18" s="30" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3589,21 +3635,21 @@
         <v>2</v>
       </c>
       <c r="B19" s="27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C19" s="27" t="inlineStr">
         <is>
-          <t>IGModel</t>
+          <t>GraphscoreDTA</t>
         </is>
       </c>
       <c r="D19" s="27" t="inlineStr">
         <is>
-          <t>models/saved_model.pth y self-ref_model.pth en el repo</t>
+          <t>model/modelp.pth en el repo + grafos CASF-2016 preparados (release Data, 35 MB)</t>
         </is>
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>PyTorch 2.2 + DGL 2.2.1 + RDKit + Open Babel 3.1.1 + spyrmsd (Python 3.10)</t>
+          <t>PyTorch 2.2 + DGL 2.2.1 (Python 3.10)</t>
         </is>
       </c>
       <c r="F19" s="28" t="inlineStr">
@@ -3626,32 +3672,32 @@
       </c>
       <c r="K19" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: test PASS: reproduce el notebook de los autores (1bcu, 10 poses, dif. 3e-6); 1a30 = 5.0653 (modo referencia; self-ref 5.4664). El .sdf de 1a30 no lo lee RDKit: usar .mol2. Eaves usa modo self-ref con saved_model.pth. Plugin: plugins/igmodel</t>
+          <t>21/10/2026: NO puede evaluar 1a30: los autores no publican el código que arma grafos y términos Vina, y 1a30 (con 2zcr, 2zy1, 3ag9, 3bv9, 3uri) no está en sus 279 complejos. El test reproduce sus 279 predicciones (dif. máx. 0.00005; PCC 0.810 en esos 279). El código original exige GPU (cuda:0). Ver tarea 6.2. Plugin: plugins/graphscoredta</t>
         </is>
       </c>
       <c r="L19" s="28" t="inlineStr">
         <is>
-          <t>igmodel</t>
+          <t>graphscoredta</t>
         </is>
       </c>
       <c r="M19" s="28" t="inlineStr">
         <is>
-          <t>demo_igmodel.bat</t>
+          <t>demo_graphscoredta.bat</t>
         </is>
       </c>
       <c r="N19" s="28" t="inlineStr">
         <is>
-          <t>combilab/igmodel:1.0</t>
+          <t>combilab/graphscoredta:1.0</t>
         </is>
       </c>
       <c r="O19" s="28" t="inlineStr">
         <is>
-          <t>docker_igmodel.bat</t>
+          <t>docker_graphscoredta.bat</t>
         </is>
       </c>
       <c r="P19" s="28" t="inlineStr">
         <is>
-          <t>docker_igmodel.sh</t>
+          <t>docker_graphscoredta.sh</t>
         </is>
       </c>
       <c r="Q19" s="30" t="inlineStr">
@@ -3670,21 +3716,21 @@
         <v>2</v>
       </c>
       <c r="B20" s="27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C20" s="27" t="inlineStr">
         <is>
-          <t>ConBAP</t>
+          <t>IGModel</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>modelo contrastivo + cabeza de afinidad repeat0 en el repo</t>
+          <t>models/saved_model.pth y self-ref_model.pth en el repo</t>
         </is>
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>PyTorch 2.2 + PyG 2.5.3 + torch_scatter/cluster + GVP-GNN + RDKit + PyMOL (Python 3.10)</t>
+          <t>PyTorch 2.2 + DGL 2.2.1 + RDKit + Open Babel 3.1.1 + spyrmsd (Python 3.10)</t>
         </is>
       </c>
       <c r="F20" s="28" t="inlineStr">
@@ -3699,7 +3745,7 @@
       </c>
       <c r="H20" s="30" t="n"/>
       <c r="I20" s="30" t="n">
-        <v>0.864</v>
+        <v>0.831</v>
       </c>
       <c r="J20" s="31">
         <f>IF(AND(ISNUMBER(H20),ISNUMBER(I20)),H20-I20,"")</f>
@@ -3707,32 +3753,32 @@
       </c>
       <c r="K20" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: test PASS: 1bcu del toy set rehecho desde cero = grafos de los autores (4.8575); 1a30 = 5.9318 con ligando sanitizado. Hallazgo: con el .sdf SIN sanitizar (como Eaves) se reproduce exacto su valor 7.7406 → probable causa de su PCC 0.424 (todas sus predicciones altas). Plugin: plugins/conbap</t>
+          <t>21/10/2026: test PASS: reproduce el notebook de los autores (1bcu, 10 poses, dif. 3e-6); 1a30 = 5.0653 (modo referencia; self-ref 5.4664). El .sdf de 1a30 no lo lee RDKit: usar .mol2. Eaves usa modo self-ref con saved_model.pth. Plugin: plugins/igmodel</t>
         </is>
       </c>
       <c r="L20" s="28" t="inlineStr">
         <is>
-          <t>conbap</t>
+          <t>igmodel</t>
         </is>
       </c>
       <c r="M20" s="28" t="inlineStr">
         <is>
-          <t>demo_conbap.bat</t>
+          <t>demo_igmodel.bat</t>
         </is>
       </c>
       <c r="N20" s="28" t="inlineStr">
         <is>
-          <t>combilab/conbap:1.0</t>
+          <t>combilab/igmodel:1.0</t>
         </is>
       </c>
       <c r="O20" s="28" t="inlineStr">
         <is>
-          <t>docker_conbap.bat</t>
+          <t>docker_igmodel.bat</t>
         </is>
       </c>
       <c r="P20" s="28" t="inlineStr">
         <is>
-          <t>docker_conbap.sh</t>
+          <t>docker_igmodel.sh</t>
         </is>
       </c>
       <c r="Q20" s="30" t="inlineStr">
@@ -3751,36 +3797,36 @@
         <v>2</v>
       </c>
       <c r="B21" s="27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C21" s="27" t="inlineStr">
         <is>
-          <t>CPIScore</t>
+          <t>ConBAP</t>
         </is>
       </c>
       <c r="D21" s="27" t="inlineStr">
         <is>
-          <t>result/model.pkl (incompleto)</t>
+          <t>modelo contrastivo + cabeza de afinidad repeat0 en el repo</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PyTorch 2.2 + PyG 2.5.3 + torch_scatter/cluster + GVP-GNN + RDKit + PyMOL (Python 3.10)</t>
         </is>
       </c>
       <c r="F21" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G21" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H21" s="30" t="n"/>
       <c r="I21" s="30" t="n">
-        <v>0.74</v>
+        <v>0.864</v>
       </c>
       <c r="J21" s="31">
         <f>IF(AND(ISNUMBER(H21),ISNUMBER(I21)),H21-I21,"")</f>
@@ -3788,89 +3834,142 @@
       </c>
       <c r="K21" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: DESCARTADA. Faltan los modelos word2vec (SMILES 256d y proteína 512d) que usan sus features, y la rama Transformer se crea con pesos aleatorios en cada forward (no está en model.pkl): predicciones no reproducibles. Ver plugins/cpiscore/INSTALL.md</t>
+          <t>21/10/2026: test PASS: 1bcu del toy set rehecho desde cero = grafos de los autores (4.8575); 1a30 = 5.9318 con ligando sanitizado. Hallazgo: con el .sdf SIN sanitizar (como Eaves) se reproduce exacto su valor 7.7406 → probable causa de su PCC 0.424 (todas sus predicciones altas). Plugin: plugins/conbap</t>
         </is>
       </c>
       <c r="L21" s="28" t="inlineStr">
         <is>
-          <t>cpiscore</t>
+          <t>conbap</t>
         </is>
       </c>
       <c r="M21" s="28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>demo_conbap.bat</t>
         </is>
       </c>
       <c r="N21" s="28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>combilab/conbap:1.0</t>
         </is>
       </c>
       <c r="O21" s="28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docker_conbap.bat</t>
         </is>
       </c>
       <c r="P21" s="28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docker_conbap.sh</t>
         </is>
       </c>
       <c r="Q21" s="30" t="inlineStr">
         <is>
-          <t>No aplica</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="R21" s="30" t="inlineStr">
         <is>
-          <t>No aplica</t>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="17">
       <c r="A22" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B22" s="27" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>PointNet</t>
-        </is>
-      </c>
-      <c r="D22" s="27" t="n"/>
+          <t>CPIScore</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>result/model.pkl (incompleto)</t>
+        </is>
+      </c>
       <c r="E22" s="27" t="inlineStr">
         <is>
-          <t>GPU / descargas grandes</t>
-        </is>
-      </c>
-      <c r="F22" s="28" t="n"/>
-      <c r="G22" s="28" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="H22" s="30" t="n"/>
-      <c r="I22" s="30" t="n"/>
+      <c r="I22" s="30" t="n">
+        <v>0.74</v>
+      </c>
       <c r="J22" s="31">
         <f>IF(AND(ISNUMBER(H22),ISNUMBER(I22)),H22-I22,"")</f>
         <v/>
       </c>
-      <c r="K22" s="28" t="n"/>
+      <c r="K22" s="28" t="inlineStr">
+        <is>
+          <t>21/10/2026: DESCARTADA. Faltan los modelos word2vec (SMILES 256d y proteína 512d) que usan sus features, y la rama Transformer se crea con pesos aleatorios en cada forward (no está en model.pkl): predicciones no reproducibles. Ver plugins/cpiscore/INSTALL.md</t>
+        </is>
+      </c>
+      <c r="L22" s="16" t="inlineStr">
+        <is>
+          <t>cpiscore</t>
+        </is>
+      </c>
+      <c r="M22" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N22" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O22" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P22" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q22" s="16" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="R22" s="16" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="17">
       <c r="A23" s="27" t="n">
         <v>3</v>
       </c>
       <c r="B23" s="27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" s="27" t="inlineStr">
         <is>
-          <t>PIGNet2</t>
+          <t>PointNet</t>
         </is>
       </c>
       <c r="D23" s="27" t="n"/>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>GPU</t>
+          <t>GPU / descargas grandes</t>
         </is>
       </c>
       <c r="F23" s="28" t="n"/>
@@ -3888,11 +3987,11 @@
         <v>3</v>
       </c>
       <c r="B24" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>Dynaformer</t>
+          <t>PIGNet2</t>
         </is>
       </c>
       <c r="D24" s="27" t="n"/>
@@ -3916,17 +4015,17 @@
         <v>3</v>
       </c>
       <c r="B25" s="27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>TopoFormer</t>
+          <t>Dynaformer</t>
         </is>
       </c>
       <c r="D25" s="27" t="n"/>
       <c r="E25" s="27" t="inlineStr">
         <is>
-          <t>GPU / descargas grandes</t>
+          <t>GPU</t>
         </is>
       </c>
       <c r="F25" s="28" t="n"/>
@@ -3944,17 +4043,17 @@
         <v>3</v>
       </c>
       <c r="B26" s="27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>BAPA</t>
+          <t>TopoFormer</t>
         </is>
       </c>
       <c r="D26" s="27" t="n"/>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>TensorFlow 1.12</t>
+          <t>GPU / descargas grandes</t>
         </is>
       </c>
       <c r="F26" s="28" t="n"/>
@@ -3972,17 +4071,17 @@
         <v>3</v>
       </c>
       <c r="B27" s="27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>CGraphDTA</t>
+          <t>BAPA</t>
         </is>
       </c>
       <c r="D27" s="27" t="n"/>
       <c r="E27" s="27" t="inlineStr">
         <is>
-          <t>Bases HHblits/BLAST</t>
+          <t>TensorFlow 1.12</t>
         </is>
       </c>
       <c r="F27" s="28" t="n"/>
@@ -4000,11 +4099,11 @@
         <v>3</v>
       </c>
       <c r="B28" s="27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C28" s="27" t="inlineStr">
         <is>
-          <t>EGNA</t>
+          <t>CGraphDTA</t>
         </is>
       </c>
       <c r="D28" s="27" t="n"/>
@@ -4028,19 +4127,19 @@
         <v>3</v>
       </c>
       <c r="B29" s="27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>HydraScreen</t>
-        </is>
-      </c>
-      <c r="D29" s="27" t="inlineStr">
-        <is>
-          <t>API con registro</t>
-        </is>
-      </c>
-      <c r="E29" s="27" t="n"/>
+          <t>EGNA</t>
+        </is>
+      </c>
+      <c r="D29" s="27" t="n"/>
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>Bases HHblits/BLAST</t>
+        </is>
+      </c>
       <c r="F29" s="28" t="n"/>
       <c r="G29" s="28" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -4056,19 +4155,19 @@
         <v>3</v>
       </c>
       <c r="B30" s="27" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>RFL-Score</t>
-        </is>
-      </c>
-      <c r="D30" s="27" t="n"/>
-      <c r="E30" s="27" t="inlineStr">
-        <is>
-          <t>Muchas herramientas</t>
-        </is>
-      </c>
+          <t>HydraScreen</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>API con registro</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="n"/>
       <c r="F30" s="28" t="n"/>
       <c r="G30" s="28" t="n"/>
       <c r="H30" s="30" t="n"/>
@@ -4084,7 +4183,7 @@
         <v>3</v>
       </c>
       <c r="B31" s="27" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C31" s="27" t="inlineStr">
         <is>
@@ -4107,7 +4206,6 @@
       </c>
       <c r="K31" s="28" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="17">
       <c r="A33" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sheet: RFL-Score Docker 1.0 failure and fix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -3348,7 +3348,7 @@
       </c>
       <c r="K15" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: SF propia de combi-lab (Arrua et al., IEEE CIBCB 2024). Test 1a30 PASS: el modelo con las 160 features de los autores (examples/1a30/1a30_160_input.csv) da 4.4494; el pipeline completo desde los archivos de CASF reproduce las 160 features EXACTAS (0 diferencias) y el mismo 4.4494. Con examples/all_160_input.csv da 4.5071 (otra versión de los descriptores RDKit 3D). Adaptaciones sin cambiar el código: wrapper de dssp para DSSP 4.2 (ya no acepta -i/-o) y prepare_ligand4.py corrido desde la carpeta del ligando. La secuencia FASTA se baja de RCSB (como los autores; incluye la cadena del péptido inhibidor); armada desde el PDB 1a30 da 4.4739. Completar PCC reportado. El RFL-Score.zip de la tabla es una versión anterior (2022), sirve para el test liviano; Docker usa el commit 2020d90. Plugin: plugins/rfl_score</t>
+          <t>21/10/2026: SF propia de combi-lab (Arrua et al., IEEE CIBCB 2024). Test 1a30 PASS: el modelo con las 160 features de los autores (examples/1a30/1a30_160_input.csv) da 4.4494; el pipeline completo desde los archivos de CASF reproduce las 160 features EXACTAS (0 diferencias) y el mismo 4.4494. Con examples/all_160_input.csv da 4.5071 (otra versión de los descriptores RDKit 3D). Adaptaciones sin cambiar el código: wrapper de dssp para DSSP 4.2 (ya no acepta -i/-o) y prepare_ligand4.py corrido desde la carpeta del ligando. La secuencia FASTA se baja de RCSB (como los autores; incluye la cadena del péptido inhibidor); armada desde el PDB 1a30 da 4.4739. Completar PCC reportado. El RFL-Score.zip de la tabla es una versión anterior (2022), sirve para el test liviano; Docker usa el commit 2020d90. Plugin: plugins/rfl_score | 21/10/2026: en la PC (Docker Desktop + WSL 2) falló con 'list index out of range': el binario estático de vina4dv (Intel, 2016) da Segmentation fault en kernels sin vsyscall (WSL 2). La imagen 1.1 compila vina4dv con g++ (salida idéntica para 1a30).</t>
         </is>
       </c>
       <c r="L15" s="28" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="N15" s="28" t="inlineStr">
         <is>
-          <t>combilab/rfl_score:1.0</t>
+          <t>combilab/rfl_score:1.1</t>
         </is>
       </c>
       <c r="O15" s="28" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="Q15" s="30" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="R15" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Sheet: RFL-Score Docker test PASS on the lab PC
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FK4FcJ1NZtPRbF4Lb6qycu
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -2332,7 +2332,7 @@
       </c>
       <c r="J35" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: test 1a30 PASS en Linux: modelo 4.4494 con las features de los autores; pipeline completo = mismas 160 features y 4.4494. Falta confirmar demo_rfl_score.bat (Windows conda) y docker_rfl_score.bat en la PC del laboratorio. El core set entra en run_coreset_level1.bat (vía Docker) para el video (8.1)</t>
+          <t>21/10/2026: test 1a30 PASS en Linux: modelo 4.4494 con las features de los autores; pipeline completo = mismas 160 features y 4.4494. Falta confirmar demo_rfl_score.bat (Windows conda) y docker_rfl_score.bat en la PC del laboratorio. El core set entra en run_coreset_level1.bat (vía Docker) para el video (8.1) | 21/10/2026: docker_rfl_score.bat PASS en la PC del laboratorio (imagen 1.1, vina4dv compilado con g++). Falta probar demo_rfl_score.bat (conda).</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="K15" s="28" t="inlineStr">
         <is>
-          <t>21/10/2026: SF propia de combi-lab (Arrua et al., IEEE CIBCB 2024). Test 1a30 PASS: el modelo con las 160 features de los autores (examples/1a30/1a30_160_input.csv) da 4.4494; el pipeline completo desde los archivos de CASF reproduce las 160 features EXACTAS (0 diferencias) y el mismo 4.4494. Con examples/all_160_input.csv da 4.5071 (otra versión de los descriptores RDKit 3D). Adaptaciones sin cambiar el código: wrapper de dssp para DSSP 4.2 (ya no acepta -i/-o) y prepare_ligand4.py corrido desde la carpeta del ligando. La secuencia FASTA se baja de RCSB (como los autores; incluye la cadena del péptido inhibidor); armada desde el PDB 1a30 da 4.4739. Completar PCC reportado. El RFL-Score.zip de la tabla es una versión anterior (2022), sirve para el test liviano; Docker usa el commit 2020d90. Plugin: plugins/rfl_score | 21/10/2026: en la PC (Docker Desktop + WSL 2) falló con 'list index out of range': el binario estático de vina4dv (Intel, 2016) da Segmentation fault en kernels sin vsyscall (WSL 2). La imagen 1.1 compila vina4dv con g++ (salida idéntica para 1a30).</t>
+          <t>21/10/2026: SF propia de combi-lab (Arrua et al., IEEE CIBCB 2024). Test 1a30 PASS: el modelo con las 160 features de los autores (examples/1a30/1a30_160_input.csv) da 4.4494; el pipeline completo desde los archivos de CASF reproduce las 160 features EXACTAS (0 diferencias) y el mismo 4.4494. Con examples/all_160_input.csv da 4.5071 (otra versión de los descriptores RDKit 3D). Adaptaciones sin cambiar el código: wrapper de dssp para DSSP 4.2 (ya no acepta -i/-o) y prepare_ligand4.py corrido desde la carpeta del ligando. La secuencia FASTA se baja de RCSB (como los autores; incluye la cadena del péptido inhibidor); armada desde el PDB 1a30 da 4.4739. Completar PCC reportado. El RFL-Score.zip de la tabla es una versión anterior (2022), sirve para el test liviano; Docker usa el commit 2020d90. Plugin: plugins/rfl_score | 21/10/2026: en la PC (Docker Desktop + WSL 2) falló con 'list index out of range': el binario estático de vina4dv (Intel, 2016) da Segmentation fault en kernels sin vsyscall (WSL 2). La imagen 1.1 compila vina4dv con g++ (salida idéntica para 1a30). | 21/10/2026: test Docker 1a30 PASS en la PC del laboratorio con la imagen 1.1 (Windows + Docker Desktop).</t>
         </is>
       </c>
       <c r="L15" s="28" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="Q15" s="30" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R15" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Add PIGNet2 plugin (Level 3, runs on CPU): 1a30 test reproduces the authors' energies; authors' 285 prepared CASF-2016 complexes give PCC 0.7467 (paper 0.747). Sheet: Level 3 review of the 9 SF
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChgNv1XU8n7w4Rues6wzrR
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1062,6 +1062,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="17">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -2136,15 +2137,17 @@
       </c>
       <c r="F30" s="28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="G30" s="28" t="n"/>
-      <c r="H30" s="29" t="n"/>
+      <c r="H30" s="29" t="n">
+        <v>46317</v>
+      </c>
       <c r="I30" s="29" t="n"/>
       <c r="J30" s="28" t="inlineStr">
         <is>
-          <t>GPU, licencias (X-Score) o API (HydraScreen)</t>
+          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final</t>
         </is>
       </c>
     </row>
@@ -2406,6 +2409,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="39" customHeight="1" s="17">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -3980,7 +3984,11 @@
         <f>IF(AND(ISNUMBER(H23),ISNUMBER(I23)),H23-I23,"")</f>
         <v/>
       </c>
-      <c r="K23" s="28" t="n"/>
+      <c r="K23" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: modelos PointNet/PointTransformer (.pth) en el repo; generación de nubes de puntos con binarios Linux (POINTNET) -&gt; Docker/WSL</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="17">
       <c r="A24" s="27" t="n">
@@ -3994,21 +4002,74 @@
           <t>PIGNet2</t>
         </is>
       </c>
-      <c r="D24" s="27" t="n"/>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>src/ckpt/pda_0..3.pt en el repo (4 modelos, se promedian)</t>
+        </is>
+      </c>
       <c r="E24" s="27" t="inlineStr">
         <is>
-          <t>GPU</t>
-        </is>
-      </c>
-      <c r="F24" s="28" t="n"/>
-      <c r="G24" s="28" t="n"/>
+          <t>PyTorch 2.2 CPU + PyG 2.0.3 + torch_scatter/sparse + RDKit 2022.03.4 + PyMOL (Python 3.9); no necesita GPU</t>
+        </is>
+      </c>
+      <c r="F24" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H24" s="30" t="n"/>
-      <c r="I24" s="30" t="n"/>
+      <c r="I24" s="30" t="n">
+        <v>0.747</v>
+      </c>
       <c r="J24" s="31">
         <f>IF(AND(ISNUMBER(H24),ISNUMBER(I24)),H24-I24,"")</f>
         <v/>
       </c>
-      <c r="K24" s="28" t="n"/>
+      <c r="K24" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: test 1a30 PASS en Linux: energías -2.865/-2.897/-3.068/-2.637 kcal/mol = las de test.py de los autores con su 1a30 preparado; pKd medio 2.1077 (exp. 4.30). Nuestra preparación de 1a30 (ligando .mol2 con H + bolsillo de generate_data.extract) es idéntica a la de los autores. Con los 285 complejos preparados por los autores (Zenodo 8091220) PCC 0.7467 (paper 0.747; Eaves 0.505). 'reduce' no hace falta (el bolsillo no lleva H). PyG 2.0.3 obligatorio. Imagen Docker sin probar (sin acceso a Docker Hub desde la máquina de prueba)</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>pignet2</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>demo_pignet2.bat</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>combilab/pignet2:1.0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>docker_pignet2.bat</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>docker_pignet2.sh</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="17">
       <c r="A25" s="27" t="n">
@@ -4036,7 +4097,11 @@
         <f>IF(AND(ISNUMBER(H25),ISNUMBER(I25)),H25-I25,"")</f>
         <v/>
       </c>
-      <c r="K25" s="28" t="n"/>
+      <c r="K25" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: checkpoints solo en OneDrive; basado en fairseq/Graphormer, solo Linux</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="17">
       <c r="A26" s="27" t="n">
@@ -4064,7 +4129,11 @@
         <f>IF(AND(ISNUMBER(H26),ISNUMBER(I26)),H26-I26,"")</f>
         <v/>
       </c>
-      <c r="K26" s="28" t="n"/>
+      <c r="K26" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: features PTHL + transformer; modelos fine-tuned en Zenodo 10892800 / weilab.math.msu.edu; PyTorch CUDA 11.7</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="17">
       <c r="A27" s="27" t="n">
@@ -4092,7 +4161,11 @@
         <f>IF(AND(ISNUMBER(H27),ISNUMBER(I27)),H27-I27,"")</f>
         <v/>
       </c>
-      <c r="K27" s="28" t="n"/>
+      <c r="K27" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: modelo TF 1.12 en el repo; necesita UCSF Chimera (pdb-&gt;mol2) y RF-Score (términos Vina) -&gt; Docker</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="17">
       <c r="A28" s="27" t="n">
@@ -4120,7 +4193,11 @@
         <f>IF(AND(ISNUMBER(H28),ISNUMBER(I28)),H28-I28,"")</f>
         <v/>
       </c>
-      <c r="K28" s="28" t="n"/>
+      <c r="K28" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: modelo en el repo, pero necesita BLAST+/UniRef90, HH-suite/Uniclust30, DSSP y Mol2vec (bases de cientos de GB)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="17">
       <c r="A29" s="27" t="n">
@@ -4148,7 +4225,11 @@
         <f>IF(AND(ISNUMBER(H29),ISNUMBER(I29)),H29-I29,"")</f>
         <v/>
       </c>
-      <c r="K29" s="28" t="n"/>
+      <c r="K29" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: 5 modelos en el repo; necesita HHblits + Uniclust30</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="17">
       <c r="A30" s="27" t="n">
@@ -4176,7 +4257,11 @@
         <f>IF(AND(ISNUMBER(H30),ISNUMBER(I30)),H30-I30,"")</f>
         <v/>
       </c>
-      <c r="K30" s="28" t="n"/>
+      <c r="K30" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: además de la API, el repo trae inferencia local (paper/model/last_model.ckpt, paper/code_release) -&gt; no haría falta registro</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="17">
       <c r="A31" s="27" t="n">
@@ -4204,8 +4289,13 @@
         <f>IF(AND(ISNUMBER(H31),ISNUMBER(I31)),H31-I31,"")</f>
         <v/>
       </c>
-      <c r="K31" s="28" t="n"/>
-    </row>
+      <c r="K31" s="28" t="inlineStr">
+        <is>
+          <t>22/10/2026: solo P3-Score_predict.py; necesita X-Score (licencia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="17">
       <c r="A33" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add PointNet/PointTransformer plugin (Level 3, CPU): 1a30 test passes (own reference values, seeded rotations); point clouds need the authors' Linux POINTNET (Docker). Sheet: HydraScreen local inference blocked by private Ro5 packages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChgNv1XU8n7w4Rues6wzrR
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -2147,7 +2147,7 @@
       <c r="I30" s="29" t="n"/>
       <c r="J30" s="28" t="inlineStr">
         <is>
-          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final</t>
+          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final | 22/10/2026: PointNet/PointTransformer hasta el test con 1a30 (PASS; pipeline completo en Docker). HydraScreen local bloqueada (paquetes privados de Ro5): queda la API</t>
         </is>
       </c>
     </row>
@@ -3970,23 +3970,72 @@
           <t>PointNet</t>
         </is>
       </c>
-      <c r="D23" s="27" t="n"/>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>5 PointTransformer + 5 PointNet (.pth) en el repo, conjunto grande (B)</t>
+        </is>
+      </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>GPU / descargas grandes</t>
-        </is>
-      </c>
-      <c r="F23" s="28" t="n"/>
-      <c r="G23" s="28" t="n"/>
+          <t>PyTorch 2.2 CPU (Python 3.10) + Open Babel; programa POINTNET (solo Linux) para la nube de puntos</t>
+        </is>
+      </c>
+      <c r="F23" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H23" s="30" t="n"/>
-      <c r="I23" s="30" t="n"/>
+      <c r="I23" s="30" t="n">
+        <v>0.859</v>
+      </c>
       <c r="J23" s="31">
         <f>IF(AND(ISNUMBER(H23),ISNUMBER(I23)),H23-I23,"")</f>
         <v/>
       </c>
       <c r="K23" s="28" t="inlineStr">
         <is>
-          <t>22/10/2026: modelos PointNet/PointTransformer (.pth) en el repo; generación de nubes de puntos con binarios Linux (POINTNET) -&gt; Docker/WSL</t>
+          <t>22/10/2026: test 1a30 PASS en Linux: nube 1a30 (Open Babel --AddPolarH + POINTNET) idéntica a la referencia; PointTransformer pKd 4.6973, PointNet 4.7429 (exp. 4.30); ejemplo de los autores 5c2h: 7.4829 / 7.5160. Valores propios (los autores no publican referencia). Rotaciones aleatorias con semilla fija. Paper: PCC 0.859 (PointTransformer) / 0.831 (PointNet), sin verificar. En Windows conda solo corren los modelos (POINTNET es Linux): pipeline completo con Docker</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>pointnet</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>demo_pointnet.bat (solo modelos)</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>combilab/pointnet:1.0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>docker_pointnet.bat</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>docker_pointnet.sh</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -4035,37 +4084,37 @@
           <t>22/10/2026: test 1a30 PASS en Linux: energías -2.865/-2.897/-3.068/-2.637 kcal/mol = las de test.py de los autores con su 1a30 preparado; pKd medio 2.1077 (exp. 4.30). Nuestra preparación de 1a30 (ligando .mol2 con H + bolsillo de generate_data.extract) es idéntica a la de los autores. Con los 285 complejos preparados por los autores (Zenodo 8091220) PCC 0.7467 (paper 0.747; Eaves 0.505). 'reduce' no hace falta (el bolsillo no lleva H). PyG 2.0.3 obligatorio. Imagen Docker sin probar (sin acceso a Docker Hub desde la máquina de prueba)</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L24" s="16" t="inlineStr">
         <is>
           <t>pignet2</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M24" s="16" t="inlineStr">
         <is>
           <t>demo_pignet2.bat</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N24" s="16" t="inlineStr">
         <is>
           <t>combilab/pignet2:1.0</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O24" s="16" t="inlineStr">
         <is>
           <t>docker_pignet2.bat</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="P24" s="16" t="inlineStr">
         <is>
           <t>docker_pignet2.sh</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="Q24" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="R24" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -4249,17 +4298,27 @@
         </is>
       </c>
       <c r="E30" s="27" t="n"/>
-      <c r="F30" s="28" t="n"/>
-      <c r="G30" s="28" t="n"/>
+      <c r="F30" s="28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="H30" s="30" t="n"/>
-      <c r="I30" s="30" t="n"/>
+      <c r="I30" s="30" t="n">
+        <v>0.86</v>
+      </c>
       <c r="J30" s="31">
         <f>IF(AND(ISNUMBER(H30),ISNUMBER(I30)),H30-I30,"")</f>
         <v/>
       </c>
       <c r="K30" s="28" t="inlineStr">
         <is>
-          <t>22/10/2026: además de la API, el repo trae inferencia local (paper/model/last_model.ckpt, paper/code_release) -&gt; no haría falta registro</t>
+          <t>22/10/2026: la inferencia local (paper/code_release + last_model.ckpt) NO se puede usar: el checkpoint y data_module.py dependen de paquetes privados de Ro5 (bio3d: ResMaxNet, MultiHead, TypesDataset; ro5utils) que no están publicados. Única vía: la API hydrascreen-api.ro5.ai (registro con email, sube los archivos a Ro5, uso no comercial). En espera de decisión</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add BAPA plugin (Level 3, CPU): reproduces the authors' 10gs example end to end (pdbqt, Vina terms, descriptors, pKd 4.91); 1a30 own reference; rf-extract from the lachrymator/RF-Score fork, prebuilt for Windows and Linux
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChgNv1XU8n7w4Rues6wzrR
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -2147,7 +2147,7 @@
       <c r="I30" s="29" t="n"/>
       <c r="J30" s="28" t="inlineStr">
         <is>
-          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final | 22/10/2026: PointNet/PointTransformer hasta el test con 1a30 (PASS; pipeline completo en Docker). HydraScreen local bloqueada (paquetes privados de Ro5): queda la API</t>
+          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final | 22/10/2026: PointNet/PointTransformer hasta el test con 1a30 (PASS; pipeline completo en Docker). HydraScreen local bloqueada (paquetes privados de Ro5): queda la API | 22/10/2026: BAPA hasta el test (PASS; reproduce el ejemplo 10gs de los autores)</t>
         </is>
       </c>
     </row>
@@ -4003,37 +4003,37 @@
           <t>22/10/2026: test 1a30 PASS en Linux: nube 1a30 (Open Babel --AddPolarH + POINTNET) idéntica a la referencia; PointTransformer pKd 4.6973, PointNet 4.7429 (exp. 4.30); ejemplo de los autores 5c2h: 7.4829 / 7.5160. Valores propios (los autores no publican referencia). Rotaciones aleatorias con semilla fija. Paper: PCC 0.859 (PointTransformer) / 0.831 (PointNet), sin verificar. En Windows conda solo corren los modelos (POINTNET es Linux): pipeline completo con Docker</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L23" s="16" t="inlineStr">
         <is>
           <t>pointnet</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M23" s="16" t="inlineStr">
         <is>
           <t>demo_pointnet.bat (solo modelos)</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="N23" s="16" t="inlineStr">
         <is>
           <t>combilab/pointnet:1.0</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O23" s="16" t="inlineStr">
         <is>
           <t>docker_pointnet.bat</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="P23" s="16" t="inlineStr">
         <is>
           <t>docker_pointnet.sh</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="Q23" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="R23" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -4196,23 +4196,72 @@
           <t>BAPA</t>
         </is>
       </c>
-      <c r="D27" s="27" t="n"/>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>module/network/BAPA_network.* en el repo (TensorFlow 1)</t>
+        </is>
+      </c>
       <c r="E27" s="27" t="inlineStr">
         <is>
-          <t>TensorFlow 1.12</t>
-        </is>
-      </c>
-      <c r="F27" s="28" t="n"/>
-      <c r="G27" s="28" t="n"/>
+          <t>TensorFlow 1.12 CPU + Open Babel 2.4.1 (Python 3.6) + rf-extract (RF-Score, fork lachrymator; binarios en plugins/bapa/bin)</t>
+        </is>
+      </c>
+      <c r="F27" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H27" s="30" t="n"/>
-      <c r="I27" s="30" t="n"/>
+      <c r="I27" s="30" t="n">
+        <v>0.819</v>
+      </c>
       <c r="J27" s="31">
         <f>IF(AND(ISNUMBER(H27),ISNUMBER(I27)),H27-I27,"")</f>
         <v/>
       </c>
       <c r="K27" s="28" t="inlineStr">
         <is>
-          <t>22/10/2026: modelo TF 1.12 en el repo; necesita UCSF Chimera (pdb-&gt;mol2) y RF-Score (términos Vina) -&gt; Docker</t>
+          <t>22/10/2026: test PASS en Linux: el ejemplo 10gs de los autores se reproduce completo (pdbqt idénticos, términos Vina, conteo de descriptores = dataset.pkl, pKd 4.91 = result.csv). 1a30 con el protein.mol2 de CASF: pKd 5.5433 (exp. 4.30), valor propio. Open Babel 2.4.1 obligatorio (OB 3 cambia el término hidrofóbico). Los autores hacen el mol2 de la proteína con UCSF Chimera: opción --protein-mol2 chimera; por defecto se usa el mol2 de CASF. Repo original de RF-Score borrado: se usa el fork lachrymator/RF-Score (mismos valores); rf-extract.exe compilado con MinGW y probado con Wine</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>bapa</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>demo_bapa.bat</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>combilab/bapa:1.0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>docker_bapa.bat</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>docker_bapa.sh</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sheet: TopoFormer and Dynaformer need manual model downloads (weilab.math.msu.edu, OneDrive)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChgNv1XU8n7w4Rues6wzrR
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1062,7 +1062,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="17">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -4148,7 +4147,7 @@
       </c>
       <c r="K25" s="28" t="inlineStr">
         <is>
-          <t>22/10/2026: checkpoints solo en OneDrive; basado en fairseq/Graphormer, solo Linux</t>
+          <t>22/10/2026: checkpoints model1-3.pt solo en OneDrive (link en checkpoint/README.md), no accesible desde las máquinas de prueba. Falta descargarlos a mano. Basado en fairseq/Graphormer (solo Linux -&gt; Docker); además trae predicciones de los autores en CASF-2016 para comparar</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4179,7 @@
       </c>
       <c r="K26" s="28" t="inlineStr">
         <is>
-          <t>22/10/2026: features PTHL + transformer; modelos fine-tuned en Zenodo 10892800 / weilab.math.msu.edu; PyTorch CUDA 11.7</t>
+          <t>22/10/2026: los 3 modelos fine-tuned para CASF-2016 (finetuned_casf2016_3models.tar.gz) y los pre-entrenados están solo en weilab.math.msu.edu, que no es accesible desde las máquinas de prueba (Zenodo 10892800 solo tiene el código). Falta descargarlos a mano o habilitar el dominio. PyTorch + transformers; features PTHL propias</t>
         </is>
       </c>
     </row>
@@ -4229,37 +4228,37 @@
           <t>22/10/2026: test PASS en Linux: el ejemplo 10gs de los autores se reproduce completo (pdbqt idénticos, términos Vina, conteo de descriptores = dataset.pkl, pKd 4.91 = result.csv). 1a30 con el protein.mol2 de CASF: pKd 5.5433 (exp. 4.30), valor propio. Open Babel 2.4.1 obligatorio (OB 3 cambia el término hidrofóbico). Los autores hacen el mol2 de la proteína con UCSF Chimera: opción --protein-mol2 chimera; por defecto se usa el mol2 de CASF. Repo original de RF-Score borrado: se usa el fork lachrymator/RF-Score (mismos valores); rf-extract.exe compilado con MinGW y probado con Wine</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L27" s="16" t="inlineStr">
         <is>
           <t>bapa</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M27" s="16" t="inlineStr">
         <is>
           <t>demo_bapa.bat</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="N27" s="16" t="inlineStr">
         <is>
           <t>combilab/bapa:1.0</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O27" s="16" t="inlineStr">
         <is>
           <t>docker_bapa.bat</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" s="16" t="inlineStr">
         <is>
           <t>docker_bapa.sh</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q27" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="R27" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>

</xml_diff>

<commit_message>
Sheet: the 10 Level 1 SF (Lista 1) pass the 1a30 test on the lab PC with Windows conda and Docker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MM3eYjxccZP8nZheBw2WKB
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1236,7 +1236,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="22">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -2193,7 +2192,7 @@
       </c>
       <c r="J27" s="34" t="inlineStr">
         <is>
-          <t>19/10/2026: PLANET pasa el test con 1a30 | 20/10/2026: egGNN (5.1040), GIGN (media 5.7230), EHIGN-PLA (media 5.4670), saCNN (5.0950) y DEAttentionDTA (6.2026 CASF / 6.3185 autores) pasan el test con 1a30 en Linux. Falta confirmar en Windows</t>
+          <t>19/10/2026: PLANET pasa el test con 1a30 | 20/10/2026: egGNN (5.1040), GIGN (media 5.7230), EHIGN-PLA (media 5.4670), saCNN (5.0950) y DEAttentionDTA (6.2026 CASF / 6.3185 autores) pasan el test con 1a30 en Linux. Falta confirmar en Windows | 25/10/2026: confirmadas en Windows (demo conda y Docker) las 10 SF del Nivel 1 de la lista original: arreglos libcurl4 (egGNN, GIGN, EHIGN-PLA, IGModel) y Open Babel (saCNN)</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2830,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="39" customHeight="1" s="22">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -2971,7 +2969,7 @@
       </c>
       <c r="K5" s="34" t="inlineStr">
         <is>
-          <t>19/10/2026: test 1a30 PASS (pKd 5.6837, igual a los autores). Requiere Python 3.7 + sklearn 0.22.2 exactos; con 0.22.2 los autores reportan PCC 0.793. Plugin: plugins/et_score</t>
+          <t>19/10/2026: test 1a30 PASS (pKd 5.6837, igual a los autores). Requiere Python 3.7 + sklearn 0.22.2 exactos; con 0.22.2 los autores reportan PCC 0.793. Plugin: plugins/et_score | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio.</t>
         </is>
       </c>
       <c r="L5" s="34" t="inlineStr">
@@ -3001,12 +2999,12 @@
       </c>
       <c r="Q5" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R5" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S5" s="33" t="inlineStr">
@@ -3057,7 +3055,7 @@
       </c>
       <c r="K6" s="34" t="inlineStr">
         <is>
-          <t>19/10/2026: test 1a30 PASS (pKd 5.6171). El repo no trae script de predicción: el modelo usa 104 features filtradas y normalizadas (tabla reconstruida desde total_set_2019.csv). generate_features.py público subcuenta los H de la proteína; corregido leyendo el elemento del PDB. Plugin: plugins/gb_score</t>
+          <t>19/10/2026: test 1a30 PASS (pKd 5.6171). El repo no trae script de predicción: el modelo usa 104 features filtradas y normalizadas (tabla reconstruida desde total_set_2019.csv). generate_features.py público subcuenta los H de la proteína; corregido leyendo el elemento del PDB. Plugin: plugins/gb_score | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio.</t>
         </is>
       </c>
       <c r="L6" s="34" t="inlineStr">
@@ -3087,12 +3085,12 @@
       </c>
       <c r="Q6" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R6" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S6" s="33" t="inlineStr">
@@ -3143,7 +3141,7 @@
       </c>
       <c r="K7" s="34" t="inlineStr">
         <is>
-          <t>19/10/2026: test 1a30 PASS. TensorFlow 2.3.4 CPU + sklearn 0.22.1 + Open Babel (ligando .mol2 -&gt; .pdb). Las aguas cristalográficas del PDB cambian la predicción (con aguas 5.4568, CASF sin aguas 5.8866): definir qué archivos usar para el PCC. Eaves et al. reproducen PCC 0.851. Plugin: plugins/onionnet2</t>
+          <t>19/10/2026: test 1a30 PASS. TensorFlow 2.3.4 CPU + sklearn 0.22.1 + Open Babel (ligando .mol2 -&gt; .pdb). Las aguas cristalográficas del PDB cambian la predicción (con aguas 5.4568, CASF sin aguas 5.8866): definir qué archivos usar para el PCC. Eaves et al. reproducen PCC 0.851. Plugin: plugins/onionnet2 | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio.</t>
         </is>
       </c>
       <c r="L7" s="34" t="inlineStr">
@@ -3173,12 +3171,12 @@
       </c>
       <c r="Q7" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R7" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S7" s="33" t="inlineStr">
@@ -3229,7 +3227,7 @@
       </c>
       <c r="K8" s="34" t="inlineStr">
         <is>
-          <t>19/10/2026: test 1a30 PASS: pKd 5.4721 idéntico a Sfcnn_2016_test.csv de los autores y 74 poses de docking iguales a test/output2 (dif. máx 0.0007). build_model() carga los pesos desde la carpeta actual. Eaves et al. reproducen PCC 0.789. Plugin: plugins/sfcnn</t>
+          <t>19/10/2026: test 1a30 PASS: pKd 5.4721 idéntico a Sfcnn_2016_test.csv de los autores y 74 poses de docking iguales a test/output2 (dif. máx 0.0007). build_model() carga los pesos desde la carpeta actual. Eaves et al. reproducen PCC 0.789. Plugin: plugins/sfcnn | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio.</t>
         </is>
       </c>
       <c r="L8" s="34" t="inlineStr">
@@ -3259,12 +3257,12 @@
       </c>
       <c r="Q8" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R8" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S8" s="33" t="inlineStr">
@@ -3315,7 +3313,7 @@
       </c>
       <c r="K9" s="34" t="inlineStr">
         <is>
-          <t>19/10/2026: test 1a30 PASS (5.8930 con core.tar.bz2 de los autores; 5.6216 con CASF .mol2). El .sdf de CASF de 1a30 no lo lee RDKit: usar core.tar.bz2 de los autores. demo/result.csv es de 2022 (modelo viejo), no sirve de referencia. Plugin: plugins/planet</t>
+          <t>19/10/2026: test 1a30 PASS (5.8930 con core.tar.bz2 de los autores; 5.6216 con CASF .mol2). El .sdf de CASF de 1a30 no lo lee RDKit: usar core.tar.bz2 de los autores. demo/result.csv es de 2022 (modelo viejo), no sirve de referencia. Plugin: plugins/planet | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio.</t>
         </is>
       </c>
       <c r="L9" s="34" t="inlineStr">
@@ -3345,12 +3343,12 @@
       </c>
       <c r="Q9" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R9" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S9" s="33" t="inlineStr">
@@ -3401,7 +3399,7 @@
       </c>
       <c r="K10" s="34" t="inlineStr">
         <is>
-          <t>20/10/2026: test 1a30 PASS (pKd 5.1040 con pocket, idéntico a Eaves et al.; 6.5326 con proteína completa). Usar _pocket.pdb: con la proteína completa Eaves obtiene PCC 0.071, con el pocket 0.669 (no reproduce el 0.86 del artículo). Ligando como SMILES desde el .mol2. El checkpoint es un modelo pickleado con clases __main__.*: el wrapper las redirige. Plugin: plugins/eggnn</t>
+          <t>20/10/2026: test 1a30 PASS (pKd 5.1040 con pocket, idéntico a Eaves et al.; 6.5326 con proteína completa). Usar _pocket.pdb: con la proteína completa Eaves obtiene PCC 0.071, con el pocket 0.669 (no reproduce el 0.86 del artículo). Ligando como SMILES desde el .mol2. El checkpoint es un modelo pickleado con clases __main__.*: el wrapper las redirige. Plugin: plugins/eggnn | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio; imagen Docker sin libcurl.so.4 (lo pide torchdata 0.8.0): se agrega libcurl4 al Dockerfile.</t>
         </is>
       </c>
       <c r="L10" s="34" t="inlineStr">
@@ -3431,12 +3429,12 @@
       </c>
       <c r="Q10" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R10" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S10" s="33" t="inlineStr">
@@ -3487,7 +3485,7 @@
       </c>
       <c r="K11" s="34" t="inlineStr">
         <is>
-          <t>20/10/2026: test 1a30 PASS (modelos 4.3883 / 6.3427 / 6.4380, media 5.7230, igual a los scripts de los autores). Nuestro grafo de 1a30 es idéntico al preparado por los autores (Zenodo 7490623); con sus 285 grafos del core set: PCC 0.844 / 0.843 / 0.832, 0.855 con la media. Pocket con PyMOL a 5 Å + obabel -d. Eaves et al. reproducen PCC 0.85. Plugin: plugins/gign</t>
+          <t>20/10/2026: test 1a30 PASS (modelos 4.3883 / 6.3427 / 6.4380, media 5.7230, igual a los scripts de los autores). Nuestro grafo de 1a30 es idéntico al preparado por los autores (Zenodo 7490623); con sus 285 grafos del core set: PCC 0.844 / 0.843 / 0.832, 0.855 con la media. Pocket con PyMOL a 5 Å + obabel -d. Eaves et al. reproducen PCC 0.85. Plugin: plugins/gign | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio; Dockerfile con libcurl4 (torchdata 0.8.0).</t>
         </is>
       </c>
       <c r="L11" s="34" t="inlineStr">
@@ -3517,12 +3515,12 @@
       </c>
       <c r="Q11" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R11" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S11" s="33" t="inlineStr">
@@ -3573,7 +3571,7 @@
       </c>
       <c r="K12" s="34" t="inlineStr">
         <is>
-          <t>20/10/2026: test 1a30 PASS (5.5024 / 5.8087 / 5.0898, media 5.4670, igual a los scripts de los autores). Código para DGL 0.9: copy_src mapeado a copy_u; el modelo modifica el grafo, se recarga por modelo. Falta calcular el PCC del core set. Eaves et al. reproducen PCC 0.851. Plugin: plugins/ehign_pla</t>
+          <t>20/10/2026: test 1a30 PASS (5.5024 / 5.8087 / 5.0898, media 5.4670, igual a los scripts de los autores). Código para DGL 0.9: copy_src mapeado a copy_u; el modelo modifica el grafo, se recarga por modelo. Falta calcular el PCC del core set. Eaves et al. reproducen PCC 0.851. Plugin: plugins/ehign_pla | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio; Dockerfile con libcurl4 (torchdata 0.8.0).</t>
         </is>
       </c>
       <c r="L12" s="34" t="inlineStr">
@@ -3603,12 +3601,12 @@
       </c>
       <c r="Q12" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R12" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S12" s="33" t="inlineStr">
@@ -3659,7 +3657,7 @@
       </c>
       <c r="K13" s="34" t="inlineStr">
         <is>
-          <t>20/10/2026: test 1a30 PASS (pKd 5.0950, idéntico a Eaves et al.; 3jvr 4.7484 y features iguales a los de los autores). No requiere HTMD (htmd 2.0.6 pide acemd3 no público): se usa moleculekit 1.11.5 con la preparación corregida de Eaves, sin el fallback HTMD/CHARMM. Checkpoint guardado en GPU, se carga en CPU. Eaves et al. reproducen PCC 0.862. Plugin: plugins/sacnn</t>
+          <t>20/10/2026: test 1a30 PASS (pKd 5.0950, idéntico a Eaves et al.; 3jvr 4.7484 y features iguales a los de los autores). No requiere HTMD (htmd 2.0.6 pide acemd3 no público): se usa moleculekit 1.11.5 con la preparación corregida de Eaves, sin el fallback HTMD/CHARMM. Checkpoint guardado en GPU, se carga en CPU. Eaves et al. reproducen PCC 0.862. Plugin: plugins/sacnn | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio; al entorno conda y a la imagen les faltaba Open Babel (el atom typer de moleculekit importa openbabel.pybel; fallaba con un .csv temporal inexistente): se agrega openbabel=3.1.1.</t>
         </is>
       </c>
       <c r="L13" s="34" t="inlineStr">
@@ -3689,12 +3687,12 @@
       </c>
       <c r="Q13" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R13" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S13" s="33" t="inlineStr">
@@ -3745,7 +3743,7 @@
       </c>
       <c r="K14" s="34" t="inlineStr">
         <is>
-          <t>20/10/2026: test 1a30 PASS (6.3185 con los datos preprocesados de los autores, igual a su kfold_result.csv; 6.2026 con archivos CASF: mismo SMILES y secuencia, pocket CASF 51 vs 56 residuos). Con los datos de los autores reproduce su kfold_result.csv en 278 complejos (PCC 0.853). Los pocket de CASF no tienen cadena: el wrapper asigna cada residuo por número y nombre en orden (A y luego B). Eaves et al. reproducen PCC 0.819. Plugin: plugins/deattentiondta</t>
+          <t>20/10/2026: test 1a30 PASS (6.3185 con los datos preprocesados de los autores, igual a su kfold_result.csv; 6.2026 con archivos CASF: mismo SMILES y secuencia, pocket CASF 51 vs 56 residuos). Con los datos de los autores reproduce su kfold_result.csv en 278 complejos (PCC 0.853). Los pocket de CASF no tienen cadena: el wrapper asigna cada residuo por número y nombre en orden (A y luego B). Eaves et al. reproducen PCC 0.819. Plugin: plugins/deattentiondta | 25/10/2026: demo Windows conda y Docker PASS en la PC del laboratorio.</t>
         </is>
       </c>
       <c r="L14" s="34" t="inlineStr">
@@ -3775,12 +3773,12 @@
       </c>
       <c r="Q14" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R14" s="37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S14" s="33" t="inlineStr">
@@ -4259,7 +4257,7 @@
       </c>
       <c r="K20" s="34" t="inlineStr">
         <is>
-          <t>21/10/2026: test PASS: reproduce el notebook de los autores (1bcu, 10 poses, dif. 3e-6); 1a30 = 5.0653 (modo referencia; self-ref 5.4664). El .sdf de 1a30 no lo lee RDKit: usar .mol2. Eaves usa modo self-ref con saved_model.pth. Plugin: plugins/igmodel</t>
+          <t>21/10/2026: test PASS: reproduce el notebook de los autores (1bcu, 10 poses, dif. 3e-6); 1a30 = 5.0653 (modo referencia; self-ref 5.4664). El .sdf de 1a30 no lo lee RDKit: usar .mol2. Eaves usa modo self-ref con saved_model.pth. Plugin: plugins/igmodel | 25/10/2026: Dockerfile con libcurl4 (torchdata 0.8.0 pide libcurl.so.4; mismo fallo que egGNN). Falta probar en la PC.</t>
         </is>
       </c>
       <c r="L20" s="34" t="inlineStr">

</xml_diff>

<commit_message>
Lista 2 Level 3 review: repos found; PLiSAGE, TransScore and GITK discarded, SST not applicable; DTA-GTOmega and DBGT-PLA wait for downloads. Add docs/LISTA_TESTS_PENDIENTES.md; docker_test_all covers every plugin
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KW7qBhYGexeTE6bXkcYVFN
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -1236,6 +1236,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="22">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -2320,7 +2321,7 @@
       <c r="I30" s="35" t="n"/>
       <c r="J30" s="34" t="inlineStr">
         <is>
-          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final | 22/10/2026: PointNet/PointTransformer hasta el test con 1a30 (PASS; pipeline completo en Docker). HydraScreen local bloqueada (paquetes privados de Ro5): queda la API | 22/10/2026: BAPA hasta el test (PASS; reproduce el ejemplo 10gs de los autores)</t>
+          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final | 22/10/2026: PointNet/PointTransformer hasta el test con 1a30 (PASS; pipeline completo en Docker). HydraScreen local bloqueada (paquetes privados de Ro5): queda la API | 22/10/2026: BAPA hasta el test (PASS; reproduce el ejemplo 10gs de los autores) | 26/10/2026: Dynaformer y TopoFormer siguen bloqueadas por la descarga de modelos (OneDrive y weilab.math.msu.edu no accesibles desde la nube ni desde la PC)</t>
         </is>
       </c>
     </row>
@@ -2539,18 +2540,18 @@
           <t>Completada</t>
         </is>
       </c>
-      <c r="G36" s="36" t="n">
-        <v>46318</v>
-      </c>
+      <c r="G36" s="36" t="n"/>
       <c r="H36" s="35" t="n">
         <v>46318</v>
       </c>
-      <c r="I36" s="35" t="inlineStr">
+      <c r="I36" s="35" t="n">
+        <v>46318</v>
+      </c>
+      <c r="J36" s="34" t="inlineStr">
         <is>
           <t>23/10/2026: agregadas a "Estado SF" con Lista = 2. CPIScore y DeepTGIN ya estaban en la Lista 1</t>
         </is>
       </c>
-      <c r="J36" s="34" t="n"/>
     </row>
     <row r="37" ht="153" customHeight="1" s="22">
       <c r="A37" s="33" t="inlineStr">
@@ -2580,17 +2581,19 @@
       </c>
       <c r="F37" s="34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G37" s="34" t="n"/>
       <c r="H37" s="35" t="n"/>
-      <c r="I37" s="35" t="inlineStr">
-        <is>
-          <t>Faltan las URL de DTA-GTOmega, PLiSAGE, TransScore, SST, DBGT-PLA y GITK (referencias de la revisión)</t>
-        </is>
-      </c>
-      <c r="J37" s="34" t="n"/>
+      <c r="I37" s="35" t="n">
+        <v>46321</v>
+      </c>
+      <c r="J37" s="34" t="inlineStr">
+        <is>
+          <t>26/10/2026: URL encontradas: DTA-GTOmega github.com/ljquanlab/DTA-GTOmega, PLiSAGE github.com/PullRequestPanda/PLiSAGE, TransScore github.com/CSUBioGroup/TransScore, SST Zenodo 10795400 (Simple SMILES Transformer, sin repo de código), DBGT-PLA github.com/wangwying/DBGT-PLA, GITK github.com/Listen-lei/GITK</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="115.5" customHeight="1" s="22">
       <c r="A38" s="33" t="inlineStr">
@@ -2623,18 +2626,18 @@
           <t>Completada</t>
         </is>
       </c>
-      <c r="G38" s="36" t="n">
-        <v>46318</v>
-      </c>
+      <c r="G38" s="36" t="n"/>
       <c r="H38" s="35" t="n">
         <v>46318</v>
       </c>
-      <c r="I38" s="35" t="inlineStr">
-        <is>
-          <t>Los de Nivel 3 "por verificar" pueden bajar de nivel cuando se revise su repo</t>
-        </is>
-      </c>
-      <c r="J38" s="34" t="n"/>
+      <c r="I38" s="35" t="n">
+        <v>46318</v>
+      </c>
+      <c r="J38" s="34" t="inlineStr">
+        <is>
+          <t>Los de Nivel 3 "por verificar" pueden bajar de nivel cuando se revise su repo | 26/10/2026: revisados los repos: PLiSAGE, TransScore y GITK descartadas (sin modelo entrenado para afinidad); SST no aplica (solo ligando, receptores de SARS-CoV-2). Quedan en Nivel 3: DTA-GTOmega y DBGT-PLA</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="26.25" customHeight="1" s="22">
       <c r="A39" s="33" t="inlineStr">
@@ -2752,13 +2755,19 @@
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="G41" s="34" t="n"/>
-      <c r="H41" s="35" t="n"/>
+      <c r="H41" s="35" t="n">
+        <v>46321</v>
+      </c>
       <c r="I41" s="35" t="n"/>
-      <c r="J41" s="34" t="n"/>
+      <c r="J41" s="34" t="inlineStr">
+        <is>
+          <t>26/10/2026: revisadas las 6. Viables: DTA-GTOmega (falta descargar pesos de OmegaFold, helixon.s3.amazonaws.com) y DBGT-PLA (faltan los grafos IChem pdbbind.tgz, bioinfo-pharma.u-strasbg.fr). Ambos dominios están bloqueados desde la nube y desde la PC. Descartadas: PLiSAGE, TransScore, GITK; SST no aplica</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:J33"/>
@@ -4673,7 +4682,7 @@
       </c>
       <c r="K25" s="34" t="inlineStr">
         <is>
-          <t>22/10/2026: checkpoints model1-3.pt solo en OneDrive (link en checkpoint/README.md), no accesible desde las máquinas de prueba. Falta descargarlos a mano. Basado en fairseq/Graphormer (solo Linux -&gt; Docker); además trae predicciones de los autores en CASF-2016 para comparar</t>
+          <t>22/10/2026: checkpoints model1-3.pt solo en OneDrive (link en checkpoint/README.md), no accesible desde las máquinas de prueba. Falta descargarlos a mano. Basado en fairseq/Graphormer (solo Linux -&gt; Docker); además trae predicciones de los autores en CASF-2016 para comparar | 26/10/2026: Reintentado: 1drv.ms/OneDrive bloqueado desde la nube y desde la PC. El fork de Eaves et al. (jeavesj/Dynaformer) tampoco trae los checkpoints. Opciones: habilitar el dominio o bajar model1-3.pt a mano desde el navegador.</t>
         </is>
       </c>
       <c r="Q25" s="21" t="n"/>
@@ -4712,7 +4721,7 @@
       </c>
       <c r="K26" s="34" t="inlineStr">
         <is>
-          <t>22/10/2026: los 3 modelos fine-tuned para CASF-2016 (finetuned_casf2016_3models.tar.gz) y los pre-entrenados están solo en weilab.math.msu.edu, que no es accesible desde las máquinas de prueba (Zenodo 10892800 solo tiene el código). Falta descargarlos a mano o habilitar el dominio. PyTorch + transformers; features PTHL propias</t>
+          <t>22/10/2026: los 3 modelos fine-tuned para CASF-2016 (finetuned_casf2016_3models.tar.gz) y los pre-entrenados están solo en weilab.math.msu.edu, que no es accesible desde las máquinas de prueba (Zenodo 10892800 solo tiene el código). Falta descargarlos a mano o habilitar el dominio. PyTorch + transformers; features PTHL propias | 26/10/2026: Reintentado: weilab.math.msu.edu bloqueado desde la nube y desde la PC; el fork jeavesj/TopoFormer y Zenodo 10892800 solo tienen el código. Falta finetuned_casf2016_3models.tar.gz (bajarlo a mano o habilitar el dominio).</t>
         </is>
       </c>
       <c r="Q26" s="21" t="n"/>
@@ -4876,7 +4885,7 @@
       </c>
       <c r="K29" s="34" t="inlineStr">
         <is>
-          <t>22/10/2026: 5 modelos en el repo; necesita HHblits + Uniclust30</t>
+          <t>22/10/2026: 5 modelos en el repo; necesita HHblits + Uniclust30 | 26/10/2026: El fork jeavesj/EGNA tampoco trae perfiles HHblits precalculados. Para el test 1a30 alcanza con el .hhm de la secuencia de 1a30 (se puede generar en el servidor web HHblits del MPI Toolkit).</t>
         </is>
       </c>
       <c r="Q29" s="21" t="n"/>
@@ -5329,12 +5338,12 @@
       </c>
       <c r="D36" s="33" t="inlineStr">
         <is>
-          <t>Por verificar (repo a completar con la referencia [26] de la revisión)</t>
+          <t>saved_pth/Davis_repr en el repo (33 modelos, Davis: quinasas) + BindingDB_repr.zip en Google Drive; NO hay modelo entrenado con PDBbind</t>
         </is>
       </c>
       <c r="E36" s="33" t="inlineStr">
         <is>
-          <t>OmegaFold (estructura de la proteína predicha, GPU) + Graph Transformers + RDKit</t>
+          <t>OmegaFold (pesos release1.pt, ~3 GB, helixon.s3.amazonaws.com) para embeddings de nodos/aristas de la proteína + mapa de contactos; PyTorch + DGL/PyG + RDKit</t>
         </is>
       </c>
       <c r="F36" s="34" t="inlineStr">
@@ -5355,7 +5364,7 @@
       </c>
       <c r="K36" s="34" t="inlineStr">
         <is>
-          <t>23/10/2026: LISTA 2, SELECCIONADA en la revisión (documentado y ejecutado). J. Mol. Biol. 2024. No encontré la URL del repo en la web: completar. Nivel 3 por OmegaFold (predice la estructura de cada proteína, pesado sin GPU). Verificar si hay modelo entrenado con PDBbind (si solo hay Davis/KIBA no sirve para CASF-2016).</t>
+          <t>26/10/2026: Repo encontrado: github.com/ljquanlab/DTA-GTOmega (commit 25f42d71) + generador de features github.com/yelujiang/OmegaFeatures. Igual que DTITR: modelos entrenados en Davis (quinasas) y BindingDB, sin estructura del complejo (FASTA + SMILES). BLOQUEADO: los pesos de OmegaFold (helixon.s3.amazonaws.com) no se pueden descargar ni desde la nube ni desde la PC (dominio fuera de la lista permitida). Con ese archivo se puede armar el test 1a30 (proteína de 99 aa, OmegaFold en CPU).</t>
         </is>
       </c>
       <c r="Q36" s="21" t="inlineStr">
@@ -5375,8 +5384,10 @@
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="22">
-      <c r="A37" s="39" t="n">
-        <v>3</v>
+      <c r="A37" s="39" t="inlineStr">
+        <is>
+          <t>Desc.</t>
+        </is>
       </c>
       <c r="B37" s="39" t="n">
         <v>11</v>
@@ -5388,12 +5399,12 @@
       </c>
       <c r="D37" s="33" t="inlineStr">
         <is>
-          <t>Por verificar (repo a completar con la referencia [41])</t>
+          <t>Solo pre_check/checkpoint.pth.tar: encoders de proteína pre-entrenados (estructura GVP + superficie MAE); sin rama del ligando ni cabeza de afinidad</t>
         </is>
       </c>
       <c r="E37" s="33" t="inlineStr">
         <is>
-          <t>Superficie molecular de la proteína + geometría 3D (herramientas de superficie, probablemente solo Linux)</t>
+          <t>PyTorch + extensiones CUDA (chamfer, EMD, pointnet2_ops); GPU de 16 GB recomendada</t>
         </is>
       </c>
       <c r="F37" s="34" t="inlineStr">
@@ -5414,17 +5425,17 @@
       </c>
       <c r="K37" s="34" t="inlineStr">
         <is>
-          <t>23/10/2026: LISTA 2. Repositorio sí, documentado sí, no ejecutado en la revisión. Nivel 3 por el cálculo de superficies. Verificar modelo entrenado y dependencias.</t>
+          <t>26/10/2026: Repo: github.com/PullRequestPanda/PLiSAGE (commit f1e6ada9; antes catly/PLiSAGE). DESCARTADA para inferencia: el checkpoint publicado es solo el pre-entrenamiento de la proteína (claves protein_struct_encoder y protein_surface_encoder); para afinidad hay que hacer el fine-tuning en PDBbind (pli_train.py), o sea reentrenar.</t>
         </is>
       </c>
       <c r="Q37" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="R37" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="S37" s="39" t="inlineStr">
@@ -5434,8 +5445,10 @@
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="22">
-      <c r="A38" s="39" t="n">
-        <v>3</v>
+      <c r="A38" s="39" t="inlineStr">
+        <is>
+          <t>Desc.</t>
+        </is>
       </c>
       <c r="B38" s="39" t="n">
         <v>12</v>
@@ -5447,12 +5460,12 @@
       </c>
       <c r="D38" s="33" t="inlineStr">
         <is>
-          <t>Por verificar (repo a completar con la referencia [13])</t>
+          <t>No publicado</t>
         </is>
       </c>
       <c r="E38" s="33" t="inlineStr">
         <is>
-          <t>Grafo del complejo + TransformerConv (PyG)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F38" s="34" t="inlineStr">
@@ -5473,17 +5486,17 @@
       </c>
       <c r="K38" s="34" t="inlineStr">
         <is>
-          <t>23/10/2026: LISTA 2. IEEE JBHI 2024 (doi 10.1109/jbhi.2024.3504851). Repositorio sí, documentado sí, no ejecutado. Nivel 3 hasta verificar si hay modelo entrenado (puede bajar a Nivel 1–2).</t>
+          <t>26/10/2026: Repo: github.com/CSUBioGroup/TransScore (commit 0320737b). DESCARTADA: el repositorio solo tiene README, CSV de etiquetas y features de entrenamiento (dataset/refined_set_affinity/feature.npz); no hay código (train.py, args.py no están) ni modelo entrenado.</t>
         </is>
       </c>
       <c r="Q38" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="R38" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="S38" s="39" t="inlineStr">
@@ -5493,8 +5506,10 @@
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="22">
-      <c r="A39" s="39" t="n">
-        <v>3</v>
+      <c r="A39" s="39" t="inlineStr">
+        <is>
+          <t>Desc.</t>
+        </is>
       </c>
       <c r="B39" s="39" t="n">
         <v>13</v>
@@ -5506,12 +5521,12 @@
       </c>
       <c r="D39" s="33" t="inlineStr">
         <is>
-          <t>Por verificar (repo a completar con la referencia [34])</t>
+          <t>Zenodo 10795400 (HPC_SurrogateDatasets.zip, 914 MB): un modelo por receptor de SARS-CoV-2 (18)</t>
         </is>
       </c>
       <c r="E39" s="33" t="inlineStr">
         <is>
-          <t>Transformers preentrenados (secuencia)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F39" s="34" t="inlineStr">
@@ -5532,17 +5547,17 @@
       </c>
       <c r="K39" s="34" t="inlineStr">
         <is>
-          <t>23/10/2026: LISTA 2. Repositorio sí, documentado sí, no ejecutado. No pude identificar el repo con certeza: completar. Nivel 3 hasta verificar modelo y entrenamiento.</t>
+          <t>26/10/2026: Identificado: SST = Simple SMILES Transformer (Vasan et al., Argonne, "High performance binding affinity prediction with a Transformer-based surrogate model", 2024). NO APLICA a CASF-2016: solo usa el SMILES del ligando y predice el puntaje de docking contra 18 receptores fijos de SARS-CoV-2; no tiene entrada de proteína ni modelo general de afinidad.</t>
         </is>
       </c>
       <c r="Q39" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="R39" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="S39" s="39" t="inlineStr">
@@ -5565,12 +5580,12 @@
       </c>
       <c r="D40" s="33" t="inlineStr">
         <is>
-          <t>Por verificar (repo a completar con la referencia [42])</t>
+          <t>models/model_GFormer_best_73_1767011167.ckpt en el repo</t>
         </is>
       </c>
       <c r="E40" s="33" t="inlineStr">
         <is>
-          <t>Grafo + Transformer (doble rama)</t>
+          <t>PyTorch + PyG (torch_sparse) + NetworkX; grafos de interacción IChem de Mastropietro et al. (pdbbind.tgz, bioinfo-pharma.u-strasbg.fr)</t>
         </is>
       </c>
       <c r="F40" s="34" t="inlineStr">
@@ -5591,7 +5606,7 @@
       </c>
       <c r="K40" s="34" t="inlineStr">
         <is>
-          <t>23/10/2026: LISTA 2. IEEE JBHI 2026 (doi 10.1109/jbhi.2026.3656542). Repositorio sí, pero sin documentación y no ejecutado. Nivel 3 por falta de documentación.</t>
+          <t>26/10/2026: Repo: github.com/wangwying/DBGT-PLA (commit 76d8a9c8), derivado de AndMastro/protein-ligand-GNN (Nat. Mach. Intell. 2023). El modelo usa grafos de interacción proteína–ligando ya calculados con IChem (8 tipos de nodo) que vienen en pdbbind.tgz del laboratorio Rognan; IChem no es público, así que solo se pueden puntuar los complejos de ese archivo. Además el MinMaxScaler de las aristas se ajusta sobre todos los grafos del dataset y el entrenamiento descarta pKd fuera de 5–11 (1a30 = 4.30 queda fuera del rango). BLOQUEADO: el dominio bioinfo-pharma.u-strasbg.fr no es accesible desde la nube ni desde la PC.</t>
         </is>
       </c>
       <c r="Q40" s="21" t="inlineStr">
@@ -5611,8 +5626,10 @@
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="22">
-      <c r="A41" s="39" t="n">
-        <v>3</v>
+      <c r="A41" s="39" t="inlineStr">
+        <is>
+          <t>Desc.</t>
+        </is>
       </c>
       <c r="B41" s="39" t="n">
         <v>15</v>
@@ -5624,12 +5641,12 @@
       </c>
       <c r="D41" s="33" t="inlineStr">
         <is>
-          <t>Por verificar (repo a completar con la referencia [14])</t>
+          <t>No publicado (main.py tiene --trained_model_path pero no hay pesos)</t>
         </is>
       </c>
       <c r="E41" s="33" t="inlineStr">
         <is>
-          <t>Por verificar</t>
+          <t>PyTorch + PyG + GRIT (basado en PSICHIC)</t>
         </is>
       </c>
       <c r="F41" s="34" t="inlineStr">
@@ -5650,17 +5667,17 @@
       </c>
       <c r="K41" s="34" t="inlineStr">
         <is>
-          <t>23/10/2026: LISTA 2. Repositorio sí, pero sin documentación y no ejecutado. Nivel 3 por falta de documentación.</t>
+          <t>26/10/2026: Repo: github.com/Listen-lei/GITK (commit c3bc711f). DESCARTADA para inferencia: no hay modelo entrenado; la carpeta de Google Drive enlazada es la de datasets de PSICHIC (sin pesos de GITK). Además predice huellas de interacción y afinidad desde secuencia; se puede usar solo reentrenando.</t>
         </is>
       </c>
       <c r="Q41" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="R41" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="S41" s="39" t="inlineStr">

</xml_diff>

<commit_message>
Add AutoDock Vina and DeltaVinaRF20 plugins (Su et al. 2019), up to the 1a30 test
AutoDock Vina (Level 1, Lista 1): engine 1.1.2 (MGLTools + Vina 1.1.2, CASF-2016 protocol)
reproduces the CASF-2016 score of 1a30 exactly (-4.99866 kcal/mol); engine 1.2.5 (Open Babel +
official Vina 1.2.5 binary, Windows) gives -4.999.
DeltaVinaRF20 (Level 2, Lista 1): authors' Python 2 feature code + vina4dv + MSMS in Docker, model
also on Windows; 1a30 = 4.7758 -> 4.78, the CASF-2016 value; authors' example 7.55.
No core set run. Sheet, README and pending-tests list updated; docker_test_all now also fails
a plugin whose log has any RESULT: FAIL.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DiJEmPzb1UDu9YGUyATb62
</commit_message>
<xml_diff>
--- a/docs/CombiLabHUB_etapas.xlsx
+++ b/docs/CombiLabHUB_etapas.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Etapas'!$A$4:$J$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Estado SF'!$A$4:$S$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Estado SF'!$A$4:$S$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -1209,7 +1209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="21" min="1" max="1"/>
@@ -1236,7 +1236,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="22">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -1663,7 +1662,11 @@
       <c r="G14" s="34" t="n"/>
       <c r="H14" s="35" t="n"/>
       <c r="I14" s="35" t="n"/>
-      <c r="J14" s="34" t="n"/>
+      <c r="J14" s="34" t="inlineStr">
+        <is>
+          <t>30/10/2026: gitlab.com sigue sin acceso desde la nube y desde la PC; DAAP y LigityScore siguen pendientes</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="22">
       <c r="A15" s="33" t="inlineStr">
@@ -2321,7 +2324,7 @@
       <c r="I30" s="35" t="n"/>
       <c r="J30" s="34" t="inlineStr">
         <is>
-          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final | 22/10/2026: PointNet/PointTransformer hasta el test con 1a30 (PASS; pipeline completo en Docker). HydraScreen local bloqueada (paquetes privados de Ro5): queda la API | 22/10/2026: BAPA hasta el test (PASS; reproduce el ejemplo 10gs de los autores) | 26/10/2026: Dynaformer y TopoFormer siguen bloqueadas por la descarga de modelos (OneDrive y weilab.math.msu.edu no accesibles desde la nube ni desde la PC)</t>
+          <t>GPU, licencias (X-Score) o API (HydraScreen) | 22/10/2026: revisadas las 9 SF. PIGNet2 hasta el test con 1a30 (PASS, corre en CPU). Orden sugerido para seguir: HydraScreen (inferencia local), PointNet, BAPA, TopoFormer, Dynaformer; CGraphDTA/EGNA (bases HHblits) y P3-Score (X-Score) al final | 22/10/2026: PointNet/PointTransformer hasta el test con 1a30 (PASS; pipeline completo en Docker). HydraScreen local bloqueada (paquetes privados de Ro5): queda la API | 22/10/2026: BAPA hasta el test (PASS; reproduce el ejemplo 10gs de los autores) | 26/10/2026: Dynaformer y TopoFormer siguen bloqueadas por la descarga de modelos (OneDrive y weilab.math.msu.edu no accesibles desde la nube ni desde la PC) | 30/10/2026: los forks de Eaves et al. (github.com/jeavesj) de TopoFormer y Dynaformer tampoco traen los checkpoints; EGNA trae los mismos 5 modelos (sigue faltando el perfil HHblits)</t>
         </is>
       </c>
     </row>
@@ -2395,7 +2398,11 @@
       <c r="G32" s="34" t="n"/>
       <c r="H32" s="35" t="n"/>
       <c r="I32" s="35" t="n"/>
-      <c r="J32" s="34" t="n"/>
+      <c r="J32" s="34" t="inlineStr">
+        <is>
+          <t>30/10/2026: revisados los forks de github.com/jeavesj. No destraban SF nuevas: LGN, MFE, aescore y CurvAGN siguen sin modelo entrenado; plip-plop (pipeline de Eaves) tiene predicciones de Dynaformer, OnionNet-2 y Pafnucy en CASF-2016</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="22">
       <c r="A33" s="33" t="inlineStr">
@@ -2766,6 +2773,94 @@
       <c r="J41" s="34" t="inlineStr">
         <is>
           <t>26/10/2026: revisadas las 6. Viables: DTA-GTOmega (falta descargar pesos de OmegaFold, helixon.s3.amazonaws.com) y DBGT-PLA (faltan los grafos IChem pdbbind.tgz, bioinfo-pharma.u-strasbg.fr). Ambos dominios están bloqueados desde la nube y desde la PC. Descartadas: PLiSAGE, TransScore, GITK; SST no aplica</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="26.25" customHeight="1" s="22">
+      <c r="A42" s="33" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="B42" s="33" t="inlineStr">
+        <is>
+          <t>5. Pruebas Nivel 1 (CPU, modelo listo)</t>
+        </is>
+      </c>
+      <c r="C42" s="33" t="inlineStr">
+        <is>
+          <t>AutoDock Vina (Su et al. 2019)</t>
+        </is>
+      </c>
+      <c r="D42" s="33" t="inlineStr">
+        <is>
+          <t>Plugin plugins/autodock_vina hasta el test con 1a30 (motores 1.1.2 y 1.2.5)</t>
+        </is>
+      </c>
+      <c r="E42" s="33" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F42" s="34" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G42" s="34" t="n"/>
+      <c r="H42" s="35" t="n">
+        <v>46325</v>
+      </c>
+      <c r="I42" s="35" t="n">
+        <v>46325</v>
+      </c>
+      <c r="J42" s="34" t="inlineStr">
+        <is>
+          <t>30/10/2026: test 1a30 PASS en Linux: Vina 1.1.2 + MGLTools reproduce exactamente el valor de CASF-2016 (-4.99866 kcal/mol); Vina 1.2.5 + Open Babel (Windows) -4.999. Falta el test en la PC del laboratorio (Windows conda y Docker). Sin core set por ahora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26.25" customHeight="1" s="22">
+      <c r="A43" s="33" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="B43" s="33" t="inlineStr">
+        <is>
+          <t>6. Pruebas Nivel 2 (pasos extra)</t>
+        </is>
+      </c>
+      <c r="C43" s="33" t="inlineStr">
+        <is>
+          <t>ΔVinaRF20 (Su et al. 2019)</t>
+        </is>
+      </c>
+      <c r="D43" s="33" t="inlineStr">
+        <is>
+          <t>Plugin plugins/deltavinarf20 hasta el test con 1a30 (features en Docker, modelo también en Windows)</t>
+        </is>
+      </c>
+      <c r="E43" s="33" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G43" s="34" t="n"/>
+      <c r="H43" s="35" t="n">
+        <v>46325</v>
+      </c>
+      <c r="I43" s="35" t="n">
+        <v>46325</v>
+      </c>
+      <c r="J43" s="34" t="inlineStr">
+        <is>
+          <t>30/10/2026: test 1a30 PASS en Linux: 4.7758 -&gt; 4.78 = CASF-2016; ejemplo de los autores 7.55. Falta el test en la PC del laboratorio (Windows conda y Docker). Sin core set por ahora.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S60"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="21" min="1" max="1"/>
@@ -5748,41 +5843,205 @@
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="22">
-      <c r="Q43" s="21" t="n"/>
-      <c r="R43" s="21" t="n"/>
+      <c r="A43" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="C43" s="33" t="inlineStr">
+        <is>
+          <t>AutoDock Vina</t>
+        </is>
+      </c>
+      <c r="D43" s="33" t="inlineStr">
+        <is>
+          <t>Ninguno (función empírica, pesos fijos). Programas: Vina 1.1.2 (bioconda) y binario oficial Vina 1.2.5 (release v1.2.5)</t>
+        </is>
+      </c>
+      <c r="E43" s="33" t="inlineStr">
+        <is>
+          <t>Windows: Python 3.10 + Open Babel 3.1.1 + vina_1.2.5_win.exe. Docker: además Vina 1.1.2 + MGLTools 1.5.7 (Python 2.7)</t>
+        </is>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G43" s="34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H43" s="37" t="n"/>
+      <c r="I43" s="37" t="n">
+        <v>0.604</v>
+      </c>
+      <c r="J43" s="38">
+        <f>IF(AND(ISNUMBER(H43),ISNUMBER(I43)),H43-I43,"")</f>
+        <v/>
+      </c>
+      <c r="K43" s="34" t="inlineStr">
+        <is>
+          <t>30/10/2026: LISTA 1 (Su et al. 2019, Funciones_Score_Su2018). Solo re-puntúa la pose cristalográfica (--score_only). Motor 1.1.2 (MGLTools + Vina 1.1.2, protocolo de CASF-2016): 1a30 = -4.99866 kcal/mol, idéntico a CASF-2016/power_scoring/examples/AutodockVina.dat. Motor 1.2.5 (Open Babel + Vina 1.2.5 --autobox, el de Windows): -4.999. pKd = -0.73349 x score (factor de ΔVinaRF20): 3.6665. Test 1a30 PASS con los dos motores en Linux (desarrollo).</t>
+        </is>
+      </c>
+      <c r="L43" s="34" t="inlineStr">
+        <is>
+          <t>autodock_vina</t>
+        </is>
+      </c>
+      <c r="M43" s="34" t="inlineStr">
+        <is>
+          <t>demo_autodock_vina.bat (Vina 1.2.5)</t>
+        </is>
+      </c>
+      <c r="N43" s="34" t="inlineStr">
+        <is>
+          <t>combilab/autodock_vina:1.0</t>
+        </is>
+      </c>
+      <c r="O43" s="34" t="inlineStr">
+        <is>
+          <t>docker_autodock_vina.bat</t>
+        </is>
+      </c>
+      <c r="P43" s="34" t="inlineStr">
+        <is>
+          <t>docker_autodock_vina.sh</t>
+        </is>
+      </c>
+      <c r="Q43" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R43" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="S43" s="33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="22">
-      <c r="A44" s="40" t="inlineStr">
-        <is>
-          <t>Descartadas (sin modelo entrenado): ECIF, MSECIF, Dowker, PerSpect ML, PPS-ML, EISA-Score, GGL-Score, MP-GNN, LGN, FGNN, MFE, MM-DRPNet, DeepTGIN (también Lista 2, ver fila), HaPPy, IMCPiDB-Score, GIaNt, CurvAGN, GCNN01, SMPLIP-Score, aescore, CPIScore (modelo incompleto, ver nota).</t>
-        </is>
-      </c>
-      <c r="Q44" s="21" t="n"/>
-      <c r="R44" s="21" t="n"/>
+      <c r="A44" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="33" t="n">
+        <v>11</v>
+      </c>
+      <c r="C44" s="33" t="inlineStr">
+        <is>
+          <t>ΔVinaRF20</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
+        <is>
+          <t>deltavina/models/rffit.rda en el repo (R randomForest, MD5 944e70f5…72cc), commit 612bbe7</t>
+        </is>
+      </c>
+      <c r="E44" s="33" t="inlineStr">
+        <is>
+          <t>Features solo Linux: código Python 2 de los autores + Open Babel 2.4.1 + MGLTools 1.5.7 + vina4dv (compilado) + MSMS 2.6.1; modelo: R + randomForest (Windows: R 4.3.3 + randomForest 4.7-1.2)</t>
+        </is>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G44" s="34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H44" s="37" t="n"/>
+      <c r="I44" s="37" t="n">
+        <v>0.8159999999999999</v>
+      </c>
+      <c r="J44" s="38">
+        <f>IF(AND(ISNUMBER(H44),ISNUMBER(I44)),H44-I44,"")</f>
+        <v/>
+      </c>
+      <c r="K44" s="34" t="inlineStr">
+        <is>
+          <t>30/10/2026: LISTA 1 (Su et al. 2019, Funciones_Score_Su2018; la mejor SF de CASF-2016). Pipeline completo en Linux: 1a30 = 4.7758 -&gt; 4.78, idéntico a CASF-2016/power_scoring/examples/deltaVinaRF20.dat (parte Vina 3.6665). Ejemplo de los autores (1a42, sus features) = 7.55 como su output.csv. Recalcular las features de 1a42 da 7.60: Open Babel 2.4.1 tipa un átomo distinto (7.38 Å² de D pasan a AR); 1a30 no se ve afectado. En Windows el test usa las features de 1a30 guardadas (features_1a30.csv). Test 1a30 PASS en Linux (desarrollo).</t>
+        </is>
+      </c>
+      <c r="L44" s="34" t="inlineStr">
+        <is>
+          <t>deltavinarf20</t>
+        </is>
+      </c>
+      <c r="M44" s="34" t="inlineStr">
+        <is>
+          <t>demo_deltavinarf20.bat (solo el modelo)</t>
+        </is>
+      </c>
+      <c r="N44" s="34" t="inlineStr">
+        <is>
+          <t>combilab/deltavinarf20:1.0</t>
+        </is>
+      </c>
+      <c r="O44" s="34" t="inlineStr">
+        <is>
+          <t>docker_deltavinarf20.bat</t>
+        </is>
+      </c>
+      <c r="P44" s="34" t="inlineStr">
+        <is>
+          <t>docker_deltavinarf20.sh</t>
+        </is>
+      </c>
+      <c r="Q44" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="R44" s="37" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="S44" s="33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="22">
-      <c r="A45" s="40" t="inlineStr">
-        <is>
-          <t>Lista 2 – descartadas: sin repositorio público (12): AffinityLM, BTDHDTA, ETransDTA, FFT-DTBA, GSDeep-DTA, GTAMP-DTA, HGTDP-DTA, MambaTransDTA, MF-CNN, PLBA-FE-DL, TransMLP-DTBA, TransVAE-DTA. Con repo pero sin modelo entrenado: MRBDTA (github.com/LiZhang30/MRBDTA, solo Davis/KIBA, secuencia + SMILES). Fuente: Apresentação.pdf (revisión sistemática de Transformers, diap. 22–23).</t>
-        </is>
-      </c>
       <c r="Q45" s="21" t="n"/>
       <c r="R45" s="21" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="22">
       <c r="A46" s="40" t="inlineStr">
         <is>
-          <t>Filas con Nivel/#/SF en verde = Lista 2. Nivel asignado el 23/10/2026 según los criterios del proyecto (1: CPU y modelo listo; 2: pasos extra; 3: pesado o por verificar).</t>
+          <t>Descartadas (sin modelo entrenado): ECIF, MSECIF, Dowker, PerSpect ML, PPS-ML, EISA-Score, GGL-Score, MP-GNN, LGN, FGNN, MFE, MM-DRPNet, DeepTGIN (también Lista 2, ver fila), HaPPy, IMCPiDB-Score, GIaNt, CurvAGN, GCNN01, SMPLIP-Score, aescore, CPIScore (modelo incompleto, ver nota).</t>
         </is>
       </c>
       <c r="Q46" s="21" t="n"/>
       <c r="R46" s="21" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="22">
+      <c r="A47" s="40" t="inlineStr">
+        <is>
+          <t>Lista 2 – descartadas: sin repositorio público (12): AffinityLM, BTDHDTA, ETransDTA, FFT-DTBA, GSDeep-DTA, GTAMP-DTA, HGTDP-DTA, MambaTransDTA, MF-CNN, PLBA-FE-DL, TransMLP-DTBA, TransVAE-DTA. Con repo pero sin modelo entrenado: MRBDTA (github.com/LiZhang30/MRBDTA, solo Davis/KIBA, secuencia + SMILES). Fuente: Apresentação.pdf (revisión sistemática de Transformers, diap. 22–23).</t>
+        </is>
+      </c>
       <c r="Q47" s="21" t="n"/>
       <c r="R47" s="21" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="22">
+      <c r="A48" s="40" t="inlineStr">
+        <is>
+          <t>Filas con Nivel/#/SF en verde = Lista 2. Nivel asignado el 23/10/2026 según los criterios del proyecto (1: CPU y modelo listo; 2: pasos extra; 3: pesado o por verificar).</t>
+        </is>
+      </c>
       <c r="Q48" s="21" t="n"/>
       <c r="R48" s="21" t="n"/>
     </row>
@@ -5834,8 +6093,16 @@
       <c r="Q60" s="21" t="n"/>
       <c r="R60" s="21" t="n"/>
     </row>
+    <row r="61">
+      <c r="Q61" s="21" t="n"/>
+      <c r="R61" s="21" t="n"/>
+    </row>
+    <row r="62">
+      <c r="Q62" s="21" t="n"/>
+      <c r="R62" s="21" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:S42"/>
+  <autoFilter ref="A4:S44"/>
   <conditionalFormatting sqref="F5:G31">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="7" text="" percent="0" bottom="0">
       <formula>"Sí"</formula>

</xml_diff>